<commit_message>
fix(excel): replace alternating row colors with white backgrounds
Use uniform white body rows and subtle horizontal separators in all daily and weekly worksheets. Preserve dark headers, filters, values, formulas and frozen panes.
</commit_message>
<xml_diff>
--- a/docs/exports/day-2026-10-17.xlsx
+++ b/docs/exports/day-2026-10-17.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="市場動向" sheetId="1" r:id="R863d578dd0fc45b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="數值明細" sheetId="2" r:id="Rfe11e92f299a42a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="欄位說明" sheetId="3" r:id="R6e052e21b100487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="市場動向" sheetId="1" r:id="R6b94f833ed9049e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="數值明細" sheetId="2" r:id="Ra0658e161b7e4912"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="欄位說明" sheetId="3" r:id="Rd6776d5bdc7b4b11"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -38,7 +38,7 @@
       <x:name val="Noto Sans CJK TC"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -50,8 +50,13 @@
         <x:fgColor rgb="FF193D34"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="4">
     <x:border>
       <x:left/>
       <x:right/>
@@ -59,11 +64,40 @@
       <x:bottom/>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFDCE4DE"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFDCE4DE"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFDCE4DE"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFDCE4DE"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="12">
+  <x:cellXfs count="22">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -84,16 +118,46 @@
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -127,7 +191,7 @@
     <x:tableColumn id="18" name="來源類型"/>
     <x:tableColumn id="19" name="來源連結"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -158,7 +222,7 @@
     <x:tableColumn id="21" name="對 AEIS 影響評估（分析）"/>
     <x:tableColumn id="22" name="來源連結"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -169,7 +233,7 @@
     <x:tableColumn id="1" name="欄位／方法"/>
     <x:tableColumn id="2" name="定義"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -452,541 +516,541 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="86.4000015258789" hidden="0" customHeight="1">
-      <x:c r="A2" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B2" s="8" t="d">
+      <x:c r="A2" s="12" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C2" s="3" t="str">
+      <x:c r="C2" s="9" t="str">
         <x:v>2026-10-17:12</x:v>
       </x:c>
-      <x:c r="D2" s="3" t="str">
+      <x:c r="D2" s="9" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E2" s="3" t="str">
+      <x:c r="E2" s="9" t="str">
         <x:v>AI 半導體；HBM；先進封裝；測試</x:v>
       </x:c>
-      <x:c r="F2" s="3" t="str">
+      <x:c r="F2" s="9" t="str">
         <x:v>晶圓製造至封裝測試</x:v>
       </x:c>
-      <x:c r="G2" s="3" t="str">
+      <x:c r="G2" s="9" t="str">
         <x:v>美光 AATT2 開幕，新增投資額未核實</x:v>
       </x:c>
-      <x:c r="H2" s="3" t="str">
+      <x:c r="H2" s="9" t="str">
         <x:v>公司描述先進封裝需求，未核實新增產量</x:v>
       </x:c>
-      <x:c r="I2" s="3" t="str">
+      <x:c r="I2" s="9" t="str">
         <x:v>美商在台廠房開幕，新增金額未披露</x:v>
       </x:c>
-      <x:c r="J2" s="3" t="str">
+      <x:c r="J2" s="9" t="str">
         <x:v>本週追蹤：AI 晶片供給要同時看 CoWoS、HBM 與後段測試</x:v>
       </x:c>
-      <x:c r="K2" s="3" t="str">
+      <x:c r="K2" s="9" t="str">
         <x:v>台積電 10 月 15 日法說表示，5 倍光罩尺寸的 CoWoS 已量產；同日美光台中 AATT2 先進封裝測試廠開幕，支援 HBM。這兩項是本週進展，今日整合追蹤，並無新增產能數字。</x:v>
       </x:c>
-      <x:c r="L2" s="3" t="str">
+      <x:c r="L2" s="9" t="str">
         <x:v>半導體設備精密電源，間接需求</x:v>
       </x:c>
-      <x:c r="M2" s="3" t="str">
+      <x:c r="M2" s="9" t="str">
         <x:v>分析：優先向設備客戶確認先進邏輯與記憶體新增設備的認證、拉貨時間及每台設備電源含量，再決定產能與備料。HBM 封裝廠開幕本身，無法證明 AEIS 獲單或收入增加。</x:v>
       </x:c>
-      <x:c r="N2" s="3" t="str">
+      <x:c r="N2" s="9" t="str">
         <x:v>近期認證與中期設備拉貨</x:v>
       </x:c>
-      <x:c r="O2" s="3" t="str">
+      <x:c r="O2" s="9" t="str">
         <x:v>確認設備客戶認證及備料節奏</x:v>
       </x:c>
-      <x:c r="P2" s="3" t="str">
+      <x:c r="P2" s="9" t="str">
         <x:v>實際產能、良率、利用率與設備訂單</x:v>
       </x:c>
-      <x:c r="Q2" s="3" t="str">
+      <x:c r="Q2" s="9" t="str">
         <x:v>高</x:v>
       </x:c>
-      <x:c r="R2" s="3" t="str">
+      <x:c r="R2" s="9" t="str">
         <x:v>First-hand</x:v>
       </x:c>
-      <x:c r="S2" s="3" t="e">
+      <x:c r="S2" s="9" t="e">
         <x:f>HYPERLINK("https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-12","完整來源與日報")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-12, friendlyName=完整來源與日報</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="86.4000015258789" hidden="0" customHeight="1">
-      <x:c r="A3" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B3" s="8" t="d">
+      <x:c r="A3" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B3" s="13" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C3" s="3" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>2026-10-17:13</x:v>
       </x:c>
-      <x:c r="D3" s="3" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E3" s="3" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>AI 資料中心；伺服器；電源；液冷</x:v>
       </x:c>
-      <x:c r="F3" s="3" t="str">
+      <x:c r="F3" s="10" t="str">
         <x:v>ODM 整機櫃至機房交付</x:v>
       </x:c>
-      <x:c r="G3" s="3" t="str">
+      <x:c r="G3" s="10" t="str">
         <x:v>產品展示，未披露新增資本支出</x:v>
       </x:c>
-      <x:c r="H3" s="3" t="str">
+      <x:c r="H3" s="10" t="str">
         <x:v>800 VDC 與液冷方案增加，出貨量未核實</x:v>
       </x:c>
-      <x:c r="I3" s="3" t="str">
+      <x:c r="I3" s="10" t="str">
         <x:v>未披露外商投資金額</x:v>
       </x:c>
-      <x:c r="J3" s="3" t="str">
+      <x:c r="J3" s="10" t="str">
         <x:v>OCP 台廠展示整機櫃、800 VDC 電源與液冷，量產驗收成為下一關</x:v>
       </x:c>
-      <x:c r="K3" s="3" t="str">
+      <x:c r="K3" s="10" t="str">
         <x:v>中央社 10 月 17 日整理 10 月 12 至 15 日 OCP 展會：緯穎、華碩與勤誠等展示下一代伺服器或機櫃，台達電、光寶與康舒展示高壓直流電源及相關方案。台達電 10 月 15 日公司稿列出 800 VDC 電源櫃、備援與液冷產品，展示規格仍需與量產部署分開。</x:v>
       </x:c>
-      <x:c r="L3" s="3" t="str">
+      <x:c r="L3" s="10" t="str">
         <x:v>資料中心電源直接相關，未證實 AEIS 新訂單</x:v>
       </x:c>
-      <x:c r="M3" s="3" t="str">
+      <x:c r="M3" s="10" t="str">
         <x:v>分析：應由雲端與 ODM 的認證時程往回排工程資源，確認功率密度、效率、可靠度、備援及供應責任。投資評估需要每櫃電源價值、量產毛利與營運資金，現有公告沒有這些可計算資料。</x:v>
       </x:c>
-      <x:c r="N3" s="3" t="str">
+      <x:c r="N3" s="10" t="str">
         <x:v>依客戶認證及量產時程</x:v>
       </x:c>
-      <x:c r="O3" s="3" t="str">
+      <x:c r="O3" s="10" t="str">
         <x:v>比較系統整合、效率與服務條件</x:v>
       </x:c>
-      <x:c r="P3" s="3" t="str">
+      <x:c r="P3" s="10" t="str">
         <x:v>認證、量產訂單與每櫃電源價值</x:v>
       </x:c>
-      <x:c r="Q3" s="3" t="str">
+      <x:c r="Q3" s="10" t="str">
         <x:v>高</x:v>
       </x:c>
-      <x:c r="R3" s="3" t="str">
+      <x:c r="R3" s="10" t="str">
         <x:v>Second-hand; First-hand</x:v>
       </x:c>
-      <x:c r="S3" s="3" t="e">
+      <x:c r="S3" s="10" t="e">
         <x:f>HYPERLINK("https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-13","完整來源與日報")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-13, friendlyName=完整來源與日報</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="86.4000015258789" hidden="0" customHeight="1">
-      <x:c r="A4" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B4" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C4" s="3" t="str">
+      <x:c r="A4" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="str">
         <x:v>2026-10-17:14</x:v>
       </x:c>
-      <x:c r="D4" s="3" t="str">
+      <x:c r="D4" s="10" t="str">
         <x:v>台灣</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="str">
+      <x:c r="E4" s="10" t="str">
         <x:v>玻璃基板；光通訊；先進封裝</x:v>
       </x:c>
-      <x:c r="F4" s="3" t="str">
+      <x:c r="F4" s="10" t="str">
         <x:v>材料零組件及製程設備</x:v>
       </x:c>
-      <x:c r="G4" s="3" t="str">
+      <x:c r="G4" s="10" t="str">
         <x:v>轉型目標，資本支出未披露</x:v>
       </x:c>
-      <x:c r="H4" s="3" t="str">
+      <x:c r="H4" s="10" t="str">
         <x:v>封裝及光通訊需求尚待認證</x:v>
       </x:c>
-      <x:c r="I4" s="3" t="str">
+      <x:c r="I4" s="10" t="str">
         <x:v>與康寧合作屬技術合作，未核實投資流入</x:v>
       </x:c>
-      <x:c r="J4" s="3" t="str">
+      <x:c r="J4" s="10" t="str">
         <x:v>友達布局玻璃基板與光通訊零組件，2030 年純面板占比目標為 30%</x:v>
       </x:c>
-      <x:c r="K4" s="3" t="str">
+      <x:c r="K4" s="10" t="str">
         <x:v>友達董事長彭双浪 10 月 17 日表示，公司在先進封裝將扮演零組件供應者，運用玻璃與 TGV 技術；與康寧合作的技術已有低軌衛星天線應用。MicroLED 光通訊與 CPO 的量產時間估計仍為兩至三年，屬公司展望。</x:v>
       </x:c>
-      <x:c r="L4" s="3" t="str">
+      <x:c r="L4" s="10" t="str">
         <x:v>新材料設備電源的潛在需求</x:v>
       </x:c>
-      <x:c r="M4" s="3" t="str">
+      <x:c r="M4" s="10" t="str">
         <x:v>分析：先辨識新材料製程使用哪些設備、是否增加電源控制要求，再決定工程投入。零組件轉型可能形成設備需求，現階段未有可量化的 AEIS 訂單或資本支出影響。</x:v>
       </x:c>
-      <x:c r="N4" s="3" t="str">
+      <x:c r="N4" s="10" t="str">
         <x:v>光通訊量產展望兩至三年，屬公司估計</x:v>
       </x:c>
-      <x:c r="O4" s="3" t="str">
+      <x:c r="O4" s="10" t="str">
         <x:v>先確認製程與可服務設備</x:v>
       </x:c>
-      <x:c r="P4" s="3" t="str">
+      <x:c r="P4" s="10" t="str">
         <x:v>客戶認證、量產良率與新業務收入</x:v>
       </x:c>
-      <x:c r="Q4" s="3" t="str">
+      <x:c r="Q4" s="10" t="str">
         <x:v>中</x:v>
       </x:c>
-      <x:c r="R4" s="3" t="str">
+      <x:c r="R4" s="10" t="str">
         <x:v>Second-hand</x:v>
       </x:c>
-      <x:c r="S4" s="3" t="e">
+      <x:c r="S4" s="10" t="e">
         <x:f>HYPERLINK("https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-14","完整來源與日報")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-14, friendlyName=完整來源與日報</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="86.4000015258789" hidden="0" customHeight="1">
-      <x:c r="A5" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B5" s="8" t="d">
+      <x:c r="A5" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B5" s="13" t="d">
         <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C5" s="3" t="str">
+      <x:c r="C5" s="10" t="str">
         <x:v>2026-10-17:15</x:v>
       </x:c>
-      <x:c r="D5" s="3" t="str">
+      <x:c r="D5" s="10" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E5" s="3" t="str">
+      <x:c r="E5" s="10" t="str">
         <x:v>終端 AI；PC；IC 設計；封裝</x:v>
       </x:c>
-      <x:c r="F5" s="3" t="str">
+      <x:c r="F5" s="10" t="str">
         <x:v>設計至品牌 PC 與企業用戶</x:v>
       </x:c>
-      <x:c r="G5" s="3" t="str">
+      <x:c r="G5" s="10" t="str">
         <x:v>新品推出，未披露新廠投資</x:v>
       </x:c>
-      <x:c r="H5" s="3" t="str">
+      <x:c r="H5" s="10" t="str">
         <x:v>公司預期本地 AI 需求，尚無售出量</x:v>
       </x:c>
-      <x:c r="I5" s="3" t="str">
+      <x:c r="I5" s="10" t="str">
         <x:v>未披露</x:v>
       </x:c>
-      <x:c r="J5" s="3" t="str">
+      <x:c r="J5" s="10" t="str">
         <x:v>RTX Spark 電腦 10 月 16 日上市，台灣設計、封裝與品牌串接終端 AI</x:v>
       </x:c>
-      <x:c r="K5" s="3" t="str">
+      <x:c r="K5" s="10" t="str">
         <x:v>NVIDIA 10 月 16 日宣布 RTX Spark Windows 電腦上市，品牌包括華碩、微星及多家國際 PC 廠，採 Grace CPU 與 Blackwell GPU。公司主管向中央社說明聯發科參與 CPU 設計，並使用 CoWoS 封裝；需求與產能判斷仍屬公司說法。</x:v>
       </x:c>
-      <x:c r="L5" s="3" t="str">
+      <x:c r="L5" s="10" t="str">
         <x:v>PC 電源與製程電源機會需分開</x:v>
       </x:c>
-      <x:c r="M5" s="3" t="str">
+      <x:c r="M5" s="10" t="str">
         <x:v>分析：分別追蹤前段設備電源、封裝設備及 PC 系統電源的可服務範圍。新品上市尚不足以調高供應量，應等待通路售出、企業導入、退貨率與平台毛利。</x:v>
       </x:c>
-      <x:c r="N5" s="3" t="str">
+      <x:c r="N5" s="10" t="str">
         <x:v>新品上市後數季</x:v>
       </x:c>
-      <x:c r="O5" s="3" t="str">
+      <x:c r="O5" s="10" t="str">
         <x:v>等待售出與企業導入，再調整供應</x:v>
       </x:c>
-      <x:c r="P5" s="3" t="str">
+      <x:c r="P5" s="10" t="str">
         <x:v>出貨、使用率、能耗與退貨率</x:v>
       </x:c>
-      <x:c r="Q5" s="3" t="str">
+      <x:c r="Q5" s="10" t="str">
         <x:v>高</x:v>
       </x:c>
-      <x:c r="R5" s="3" t="str">
+      <x:c r="R5" s="10" t="str">
         <x:v>First-hand; Second-hand</x:v>
       </x:c>
-      <x:c r="S5" s="3" t="e">
+      <x:c r="S5" s="10" t="e">
         <x:f>HYPERLINK("https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-15","完整來源與日報")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-15, friendlyName=完整來源與日報</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="86.4000015258789" hidden="0" customHeight="1">
-      <x:c r="A6" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="d">
+      <x:c r="A6" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="d">
         <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C6" s="3" t="str">
+      <x:c r="C6" s="10" t="str">
         <x:v>2026-10-17:4</x:v>
       </x:c>
-      <x:c r="D6" s="3" t="str">
+      <x:c r="D6" s="10" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E6" s="3" t="str">
+      <x:c r="E6" s="10" t="str">
         <x:v>海外工業園區；電子供應鏈</x:v>
       </x:c>
-      <x:c r="F6" s="3" t="str">
+      <x:c r="F6" s="10" t="str">
         <x:v>零組件至在地工廠</x:v>
       </x:c>
-      <x:c r="G6" s="3" t="str">
+      <x:c r="G6" s="10" t="str">
         <x:v>每座 20 億至 40 億美元估算，未承諾</x:v>
       </x:c>
-      <x:c r="H6" s="3" t="str">
+      <x:c r="H6" s="10" t="str">
         <x:v>在地供應鏈規劃，租用率未公布</x:v>
       </x:c>
-      <x:c r="I6" s="3" t="str">
+      <x:c r="I6" s="10" t="str">
         <x:v>私人籌資規劃，尚非實際投資流量</x:v>
       </x:c>
-      <x:c r="J6" s="3" t="str">
+      <x:c r="J6" s="10" t="str">
         <x:v>經濟部說明赴美園區由業者籌資，每座估 20 億至 40 億美元</x:v>
       </x:c>
-      <x:c r="K6" s="3" t="str">
+      <x:c r="K6" s="10" t="str">
         <x:v>經濟部 10 月 16 日向中央社說明，將與電電公會推動海外產業園區，採業者出資、政府協助模式。龔明鑫專訪提及由德州起步、規劃不只一座；單一園區 20 億至 40 億美元是估算，土地取得細節尚未對外確認。</x:v>
       </x:c>
-      <x:c r="L6" s="3" t="str">
+      <x:c r="L6" s="10" t="str">
         <x:v>在地服務、庫存與製造成本</x:v>
       </x:c>
-      <x:c r="M6" s="3" t="str">
+      <x:c r="M6" s="10" t="str">
         <x:v>大型客戶在美國蓋廠，只完成供應鏈在地化的一部分。對中小供應商，關鍵是園區能否提供穩定訂單、共用設施與可負擔的資金，而不只是一塊海外土地。</x:v>
       </x:c>
-      <x:c r="N6" s="3" t="str">
+      <x:c r="N6" s="10" t="str">
         <x:v>用地及融資確定後</x:v>
       </x:c>
-      <x:c r="O6" s="3" t="str">
+      <x:c r="O6" s="10" t="str">
         <x:v>以已簽需求檢查布局</x:v>
       </x:c>
-      <x:c r="P6" s="3" t="str">
+      <x:c r="P6" s="10" t="str">
         <x:v>融資、土地、入駐名單與動工</x:v>
       </x:c>
-      <x:c r="Q6" s="3" t="str">
+      <x:c r="Q6" s="10" t="str">
         <x:v>中</x:v>
       </x:c>
-      <x:c r="R6" s="3" t="str">
+      <x:c r="R6" s="10" t="str">
         <x:v>Second-hand</x:v>
       </x:c>
-      <x:c r="S6" s="3" t="e">
+      <x:c r="S6" s="10" t="e">
         <x:f>HYPERLINK("https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-4","完整來源與日報")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-4, friendlyName=完整來源與日報</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="86.4000015258789" hidden="0" customHeight="1">
-      <x:c r="A7" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B7" s="8" t="d">
+      <x:c r="A7" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B7" s="13" t="d">
         <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C7" s="3" t="str">
+      <x:c r="C7" s="10" t="str">
         <x:v>2026-10-17:11</x:v>
       </x:c>
-      <x:c r="D7" s="3" t="str">
+      <x:c r="D7" s="10" t="str">
         <x:v>台灣</x:v>
       </x:c>
-      <x:c r="E7" s="3" t="str">
+      <x:c r="E7" s="10" t="str">
         <x:v>總體經濟；AI 投資</x:v>
       </x:c>
-      <x:c r="F7" s="3" t="str">
+      <x:c r="F7" s="10" t="str">
         <x:v>需求與區域投資背景</x:v>
       </x:c>
-      <x:c r="G7" s="3" t="str">
+      <x:c r="G7" s="10" t="str">
         <x:v>中經院投資展望，屬預測</x:v>
       </x:c>
-      <x:c r="H7" s="3" t="str">
+      <x:c r="H7" s="10" t="str">
         <x:v>2026 年 GDP 成長預測 12.16%</x:v>
       </x:c>
-      <x:c r="I7" s="3" t="str">
+      <x:c r="I7" s="10" t="str">
         <x:v>未提供本期 FDI 數據</x:v>
       </x:c>
-      <x:c r="J7" s="3" t="str">
+      <x:c r="J7" s="10" t="str">
         <x:v>中經院上修台灣全年成長預測至 12.16%，需分開看實績與展望</x:v>
       </x:c>
-      <x:c r="K7" s="3" t="str">
+      <x:c r="K7" s="10" t="str">
         <x:v>中經院 10 月 16 日公布第四季預測，把 2026 年經濟成長率由 7 月的 10.35% 上修至 12.16%，提高 1.81 個百分點。預估內需貢獻 6.63 個百分點、國外淨需求貢獻 5.53 個百分點；全年數字仍是預測。</x:v>
       </x:c>
-      <x:c r="L7" s="3" t="str">
+      <x:c r="L7" s="10" t="str">
         <x:v>客戶資本支出與區域服務規劃</x:v>
       </x:c>
-      <x:c r="M7" s="3" t="str">
+      <x:c r="M7" s="10" t="str">
         <x:v>這份預測的重點是 AI 硬體需求如何傳到投資與消費。分析時仍要分清：少數出口產業的強勁成長、整體 GDP，以及每個人的收入感受，三者不會等比例變動。</x:v>
       </x:c>
-      <x:c r="N7" s="3" t="str">
+      <x:c r="N7" s="10" t="str">
         <x:v>2026 年全年預測</x:v>
       </x:c>
-      <x:c r="O7" s="3" t="str">
+      <x:c r="O7" s="10" t="str">
         <x:v>用設備客戶訂單驗證總體展望</x:v>
       </x:c>
-      <x:c r="P7" s="3" t="str">
+      <x:c r="P7" s="10" t="str">
         <x:v>GDP 實績、民間投資與客戶拉貨</x:v>
       </x:c>
-      <x:c r="Q7" s="3" t="str">
+      <x:c r="Q7" s="10" t="str">
         <x:v>高</x:v>
       </x:c>
-      <x:c r="R7" s="3" t="str">
+      <x:c r="R7" s="10" t="str">
         <x:v>First-hand; Second-hand</x:v>
       </x:c>
-      <x:c r="S7" s="3" t="e">
+      <x:c r="S7" s="10" t="e">
         <x:f>HYPERLINK("https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-11","完整來源與日報")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-11, friendlyName=完整來源與日報</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="86.4000015258789" hidden="0" customHeight="1">
-      <x:c r="A8" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B8" s="8" t="d">
+      <x:c r="A8" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B8" s="13" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C8" s="3" t="str">
+      <x:c r="C8" s="10" t="str">
         <x:v>2026-10-17:18</x:v>
       </x:c>
-      <x:c r="D8" s="3" t="str">
+      <x:c r="D8" s="10" t="str">
         <x:v>越南</x:v>
       </x:c>
-      <x:c r="E8" s="3" t="str">
+      <x:c r="E8" s="10" t="str">
         <x:v>AI 資料中心；電源；能源</x:v>
       </x:c>
-      <x:c r="F8" s="3" t="str">
+      <x:c r="F8" s="10" t="str">
         <x:v>機房建設與營運電力</x:v>
       </x:c>
-      <x:c r="G8" s="3" t="str">
+      <x:c r="G8" s="10" t="str">
         <x:v>21 億美元既有計畫，新增投資未核實</x:v>
       </x:c>
-      <x:c r="H8" s="3" t="str">
+      <x:c r="H8" s="10" t="str">
         <x:v>電價爭點可能影響進度，量化需求未知</x:v>
       </x:c>
-      <x:c r="I8" s="3" t="str">
+      <x:c r="I8" s="10" t="str">
         <x:v>AIC 與 KBC 既有計畫，非新流入</x:v>
       </x:c>
-      <x:c r="J8" s="3" t="str">
+      <x:c r="J8" s="10" t="str">
         <x:v>胡志明市要求釐清 AI 資料中心電價，投資模型面臨費率認定</x:v>
       </x:c>
-      <x:c r="K8" s="3" t="str">
+      <x:c r="K8" s="10" t="str">
         <x:v>TNGlobal 10 月 16 日報導，胡志明市工業區管理機關在 10 月 15 日經濟會議要求統一 AI 資料中心電價指引。所涉 AIC 與 KBC 計畫早於 3 月公布，總規劃金額 21 億美元；本次新增進展是電價問題，並非新宣布投資。</x:v>
       </x:c>
-      <x:c r="L8" s="3" t="str">
+      <x:c r="L8" s="10" t="str">
         <x:v>資料中心電源，部署時點風險</x:v>
       </x:c>
-      <x:c r="M8" s="3" t="str">
+      <x:c r="M8" s="10" t="str">
         <x:v>分析：先確認客戶取得的電力條件，再安排機櫃電源工程與交貨。節能、功率密度及可靠度仍有價值，但現有資料不足以估算 AEIS 收入或投資回收。</x:v>
       </x:c>
-      <x:c r="N8" s="3" t="str">
+      <x:c r="N8" s="10" t="str">
         <x:v>待費率分類與電力合約</x:v>
       </x:c>
-      <x:c r="O8" s="3" t="str">
+      <x:c r="O8" s="10" t="str">
         <x:v>確認電力條件再排工程及交貨</x:v>
       </x:c>
-      <x:c r="P8" s="3" t="str">
+      <x:c r="P8" s="10" t="str">
         <x:v>正式費率、融資與上線</x:v>
       </x:c>
-      <x:c r="Q8" s="3" t="str">
+      <x:c r="Q8" s="10" t="str">
         <x:v>中</x:v>
       </x:c>
-      <x:c r="R8" s="3" t="str">
+      <x:c r="R8" s="10" t="str">
         <x:v>Second-hand</x:v>
       </x:c>
-      <x:c r="S8" s="3" t="e">
+      <x:c r="S8" s="10" t="e">
         <x:f>HYPERLINK("https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-18","完整來源與日報")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-18, friendlyName=完整來源與日報</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="86.4000015258789" hidden="0" customHeight="1">
-      <x:c r="A9" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B9" s="8" t="d">
+      <x:c r="A9" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B9" s="13" t="d">
         <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C9" s="3" t="str">
+      <x:c r="C9" s="10" t="str">
         <x:v>2026-10-17:19</x:v>
       </x:c>
-      <x:c r="D9" s="3" t="str">
+      <x:c r="D9" s="10" t="str">
         <x:v>馬來西亞；台灣</x:v>
       </x:c>
-      <x:c r="E9" s="3" t="str">
+      <x:c r="E9" s="10" t="str">
         <x:v>半導體；後段封測；設備服務</x:v>
       </x:c>
-      <x:c r="F9" s="3" t="str">
+      <x:c r="F9" s="10" t="str">
         <x:v>設計至封測及現場工程</x:v>
       </x:c>
-      <x:c r="G9" s="3" t="str">
+      <x:c r="G9" s="10" t="str">
         <x:v>人才與園區布局，非已確認新廠投資</x:v>
       </x:c>
-      <x:c r="H9" s="3" t="str">
+      <x:c r="H9" s="10" t="str">
         <x:v>逾 1,500 職缺，非實際聘用</x:v>
       </x:c>
-      <x:c r="I9" s="3" t="str">
+      <x:c r="I9" s="10" t="str">
         <x:v>未提供新增 FDI 流量</x:v>
       </x:c>
-      <x:c r="J9" s="3" t="str">
+      <x:c r="J9" s="10" t="str">
         <x:v>馬來西亞半導體招募涵蓋製程、設備與廠務，人才連結台灣供應鏈</x:v>
       </x:c>
-      <x:c r="K9" s="3" t="str">
+      <x:c r="K9" s="10" t="str">
         <x:v>中央社 10 月 16 日報導，雪蘭莪 10 月 14 至 17 日半導體招募活動提供逾 1,500 個職缺，涵蓋設計、軟韌體、製程、設備及廠務。官員表示兩座 IC 設計園區有 20 家公司、409 名工程師，並將雪蘭莪設計與檳城製造、組裝測試視為互補。</x:v>
       </x:c>
-      <x:c r="L9" s="3" t="str">
+      <x:c r="L9" s="10" t="str">
         <x:v>區域服務與工程人才，間接相關</x:v>
       </x:c>
-      <x:c r="M9" s="3" t="str">
+      <x:c r="M9" s="10" t="str">
         <x:v>分析：區域服務布局應同時評估客戶密度、現場工程人才與維修週轉時間。台馬培訓合作值得追蹤，但本期沒有確認 AEIS 合作、客戶採購或新的工廠投資。</x:v>
       </x:c>
-      <x:c r="N9" s="3" t="str">
+      <x:c r="N9" s="10" t="str">
         <x:v>當期招募與後續認證</x:v>
       </x:c>
-      <x:c r="O9" s="3" t="str">
+      <x:c r="O9" s="10" t="str">
         <x:v>檢查客戶密度、人才與維修週轉</x:v>
       </x:c>
-      <x:c r="P9" s="3" t="str">
+      <x:c r="P9" s="10" t="str">
         <x:v>聘用、留任與客戶設備認證</x:v>
       </x:c>
-      <x:c r="Q9" s="3" t="str">
+      <x:c r="Q9" s="10" t="str">
         <x:v>中</x:v>
       </x:c>
-      <x:c r="R9" s="3" t="str">
+      <x:c r="R9" s="10" t="str">
         <x:v>Second-hand</x:v>
       </x:c>
-      <x:c r="S9" s="3" t="e">
+      <x:c r="S9" s="10" t="e">
         <x:f>HYPERLINK("https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-19","完整來源與日報")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-19, friendlyName=完整來源與日報</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="86.4000015258789" hidden="0" customHeight="1">
-      <x:c r="A10" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B10" s="8" t="d">
+      <x:c r="A10" s="14" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="d">
         <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C10" s="3" t="str">
+      <x:c r="C10" s="11" t="str">
         <x:v>2026-10-17:20</x:v>
       </x:c>
-      <x:c r="D10" s="3" t="str">
+      <x:c r="D10" s="11" t="str">
         <x:v>越南；新加坡</x:v>
       </x:c>
-      <x:c r="E10" s="3" t="str">
+      <x:c r="E10" s="11" t="str">
         <x:v>製造業；外商投資；工業電源</x:v>
       </x:c>
-      <x:c r="F10" s="3" t="str">
+      <x:c r="F10" s="11" t="str">
         <x:v>資金註冊至工廠落地</x:v>
       </x:c>
-      <x:c r="G10" s="3" t="str">
+      <x:c r="G10" s="11" t="str">
         <x:v>總註冊外資 503.6 億美元</x:v>
       </x:c>
-      <x:c r="H10" s="3" t="str">
+      <x:c r="H10" s="11" t="str">
         <x:v>工廠設備需求尚須分項驗證</x:v>
       </x:c>
-      <x:c r="I10" s="3" t="str">
+      <x:c r="I10" s="11" t="str">
         <x:v>FDI 實現額估 210.7 億美元，YoY 12.1%</x:v>
       </x:c>
-      <x:c r="J10" s="3" t="str">
+      <x:c r="J10" s="11" t="str">
         <x:v>區域背景：越南前三季 FDI 實現額年增 12.1%，註冊額與落地須分開</x:v>
       </x:c>
-      <x:c r="K10" s="3" t="str">
+      <x:c r="K10" s="11" t="str">
         <x:v>越南政府新聞網 10 月 3 日公布的前三季資料顯示，FDI 實現額估 210.7 億美元、年增 12.1%，總註冊外資為 503.6 億美元、年增 76.4%。這是本期新增的區域背景，資料截至 9 月 30 日，並非 10 月 17 日的新統計。</x:v>
       </x:c>
-      <x:c r="L10" s="3" t="str">
+      <x:c r="L10" s="11" t="str">
         <x:v>在地工業電源與服務的背景指標</x:v>
       </x:c>
-      <x:c r="M10" s="3" t="str">
+      <x:c r="M10" s="11" t="str">
         <x:v>分析：先把投資案對到具名工廠、設備進口、電網接入與驗收，再估在地工業電源及維修需求。全國 FDI 只能提供市場背景，無法直接推成半導體設備或 AEIS 的成長率。</x:v>
       </x:c>
-      <x:c r="N10" s="3" t="str">
+      <x:c r="N10" s="11" t="str">
         <x:v>截至 2026 年 9 月的區域背景</x:v>
       </x:c>
-      <x:c r="O10" s="3" t="str">
+      <x:c r="O10" s="11" t="str">
         <x:v>對到具名廠房與設備採購</x:v>
       </x:c>
-      <x:c r="P10" s="3" t="str">
+      <x:c r="P10" s="11" t="str">
         <x:v>製造業分項、電網接入與驗收</x:v>
       </x:c>
-      <x:c r="Q10" s="3" t="str">
+      <x:c r="Q10" s="11" t="str">
         <x:v>高</x:v>
       </x:c>
-      <x:c r="R10" s="3" t="str">
+      <x:c r="R10" s="11" t="str">
         <x:v>First-hand; Second-hand</x:v>
       </x:c>
-      <x:c r="S10" s="3" t="e">
+      <x:c r="S10" s="11" t="e">
         <x:f>HYPERLINK("https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-20","完整來源與日報")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://aiwlulu.github.io/daily-brief-site/?view=day&amp;date=2026-10-17#story-2026-10-17-20, friendlyName=完整來源與日報</x:v>
       </x:c>
@@ -994,7 +1058,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R182c7a99fc8a4b2a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06561fd696054592"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1099,959 +1163,959 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="72" hidden="0" customHeight="1">
-      <x:c r="A2" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B2" s="8" t="d">
+      <x:c r="A2" s="12" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C2" s="3" t="str">
+      <x:c r="C2" s="9" t="str">
         <x:v>2026-10-17:12</x:v>
       </x:c>
-      <x:c r="D2" s="3" t="str">
+      <x:c r="D2" s="9" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E2" s="3" t="str">
+      <x:c r="E2" s="9" t="str">
         <x:v>AI 半導體；HBM；先進封裝；測試</x:v>
       </x:c>
-      <x:c r="F2" s="3" t="str">
+      <x:c r="F2" s="9" t="str">
         <x:v>新台幣營收（約）</x:v>
       </x:c>
-      <x:c r="G2" s="3" t="str">
+      <x:c r="G2" s="9" t="str">
         <x:v>公司實績</x:v>
       </x:c>
-      <x:c r="H2" s="3" t="str">
+      <x:c r="H2" s="9" t="str">
         <x:v>2026 Q3</x:v>
       </x:c>
-      <x:c r="I2" s="9" t="n">
+      <x:c r="I2" s="15" t="n">
         <x:v>1494</x:v>
       </x:c>
-      <x:c r="J2" s="3" t="str">
+      <x:c r="J2" s="9" t="str">
         <x:v>NTD billion</x:v>
       </x:c>
-      <x:c r="K2" s="3" t="str">
+      <x:c r="K2" s="9" t="str">
         <x:v>2025 Q3</x:v>
       </x:c>
-      <x:c r="L2" s="9"/>
-      <x:c r="M2" s="3" t="str">
+      <x:c r="L2" s="15"/>
+      <x:c r="M2" s="9" t="str">
         <x:v>YoY</x:v>
       </x:c>
-      <x:c r="N2" s="10" t="n">
+      <x:c r="N2" s="16" t="n">
         <x:v>0.509</x:v>
       </x:c>
-      <x:c r="O2" s="10"/>
-      <x:c r="P2" s="9"/>
-      <x:c r="Q2" s="9"/>
-      <x:c r="R2" s="10"/>
-      <x:c r="S2" s="3" t="str">
+      <x:c r="O2" s="16"/>
+      <x:c r="P2" s="15"/>
+      <x:c r="Q2" s="15"/>
+      <x:c r="R2" s="16"/>
+      <x:c r="S2" s="9" t="str">
         <x:v>本期值及公布增幅已核對；本表未收錄可比基期</x:v>
       </x:c>
-      <x:c r="T2" s="3" t="str">
+      <x:c r="T2" s="9" t="str">
         <x:v>TSMC</x:v>
       </x:c>
-      <x:c r="U2" s="3" t="str">
+      <x:c r="U2" s="9" t="str">
         <x:v>分析：優先向設備客戶確認先進邏輯與記憶體新增設備的認證、拉貨時間及每台設備電源含量，再決定產能與備料。HBM 封裝廠開幕本身，無法證明 AEIS 獲單或收入增加。</x:v>
       </x:c>
-      <x:c r="V2" s="3" t="e">
+      <x:c r="V2" s="9" t="e">
         <x:f>HYPERLINK("https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf","https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf, friendlyName=https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="72" hidden="0" customHeight="1">
-      <x:c r="A3" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B3" s="8" t="d">
+      <x:c r="A3" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B3" s="13" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C3" s="3" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>2026-10-17:12</x:v>
       </x:c>
-      <x:c r="D3" s="3" t="str">
+      <x:c r="D3" s="10" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E3" s="3" t="str">
+      <x:c r="E3" s="10" t="str">
         <x:v>AI 半導體；HBM；先進封裝；測試</x:v>
       </x:c>
-      <x:c r="F3" s="3" t="str">
+      <x:c r="F3" s="10" t="str">
         <x:v>稅後淨利</x:v>
       </x:c>
-      <x:c r="G3" s="3" t="str">
+      <x:c r="G3" s="10" t="str">
         <x:v>公司實績</x:v>
       </x:c>
-      <x:c r="H3" s="3" t="str">
+      <x:c r="H3" s="10" t="str">
         <x:v>2026 Q3</x:v>
       </x:c>
-      <x:c r="I3" s="9" t="n">
+      <x:c r="I3" s="17" t="n">
         <x:v>763.06</x:v>
       </x:c>
-      <x:c r="J3" s="3" t="str">
+      <x:c r="J3" s="10" t="str">
         <x:v>NTD billion</x:v>
       </x:c>
-      <x:c r="K3" s="3" t="str">
+      <x:c r="K3" s="10" t="str">
         <x:v>2025 Q3</x:v>
       </x:c>
-      <x:c r="L3" s="9"/>
-      <x:c r="M3" s="3" t="str">
+      <x:c r="L3" s="17"/>
+      <x:c r="M3" s="10" t="str">
         <x:v>YoY</x:v>
       </x:c>
-      <x:c r="N3" s="10" t="n">
+      <x:c r="N3" s="18" t="n">
         <x:v>0.687</x:v>
       </x:c>
-      <x:c r="O3" s="10"/>
-      <x:c r="P3" s="9"/>
-      <x:c r="Q3" s="9"/>
-      <x:c r="R3" s="10"/>
-      <x:c r="S3" s="3" t="str">
+      <x:c r="O3" s="18"/>
+      <x:c r="P3" s="17"/>
+      <x:c r="Q3" s="17"/>
+      <x:c r="R3" s="18"/>
+      <x:c r="S3" s="10" t="str">
         <x:v>本期值及公布增幅已核對；本表未收錄可比基期</x:v>
       </x:c>
-      <x:c r="T3" s="3" t="str">
+      <x:c r="T3" s="10" t="str">
         <x:v>TSMC</x:v>
       </x:c>
-      <x:c r="U3" s="3" t="str">
+      <x:c r="U3" s="10" t="str">
         <x:v>分析：優先向設備客戶確認先進邏輯與記憶體新增設備的認證、拉貨時間及每台設備電源含量，再決定產能與備料。HBM 封裝廠開幕本身，無法證明 AEIS 獲單或收入增加。</x:v>
       </x:c>
-      <x:c r="V3" s="3" t="e">
+      <x:c r="V3" s="10" t="e">
         <x:f>HYPERLINK("https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf","https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf, friendlyName=https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="72" hidden="0" customHeight="1">
-      <x:c r="A4" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B4" s="8" t="d">
+      <x:c r="A4" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C4" s="3" t="str">
+      <x:c r="C4" s="10" t="str">
         <x:v>2026-10-17:12</x:v>
       </x:c>
-      <x:c r="D4" s="3" t="str">
+      <x:c r="D4" s="10" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="str">
+      <x:c r="E4" s="10" t="str">
         <x:v>AI 半導體；HBM；先進封裝；測試</x:v>
       </x:c>
-      <x:c r="F4" s="3" t="str">
+      <x:c r="F4" s="10" t="str">
         <x:v>美元營收</x:v>
       </x:c>
-      <x:c r="G4" s="3" t="str">
+      <x:c r="G4" s="10" t="str">
         <x:v>公司實績</x:v>
       </x:c>
-      <x:c r="H4" s="3" t="str">
+      <x:c r="H4" s="10" t="str">
         <x:v>2026 Q3</x:v>
       </x:c>
-      <x:c r="I4" s="9" t="n">
+      <x:c r="I4" s="17" t="n">
         <x:v>46.72</x:v>
       </x:c>
-      <x:c r="J4" s="3" t="str">
+      <x:c r="J4" s="10" t="str">
         <x:v>USD billion</x:v>
       </x:c>
-      <x:c r="K4" s="3" t="str"/>
-      <x:c r="L4" s="9"/>
-      <x:c r="M4" s="3" t="str">
+      <x:c r="K4" s="10" t="str"/>
+      <x:c r="L4" s="17"/>
+      <x:c r="M4" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N4" s="10"/>
-      <x:c r="O4" s="10"/>
-      <x:c r="P4" s="9"/>
-      <x:c r="Q4" s="9"/>
-      <x:c r="R4" s="10"/>
-      <x:c r="S4" s="3" t="str">
+      <x:c r="N4" s="18"/>
+      <x:c r="O4" s="18"/>
+      <x:c r="P4" s="17"/>
+      <x:c r="Q4" s="17"/>
+      <x:c r="R4" s="18"/>
+      <x:c r="S4" s="10" t="str">
         <x:v>本期值及公布增幅已核對；本表未收錄可比基期</x:v>
       </x:c>
-      <x:c r="T4" s="3" t="str">
+      <x:c r="T4" s="10" t="str">
         <x:v>TSMC</x:v>
       </x:c>
-      <x:c r="U4" s="3" t="str">
+      <x:c r="U4" s="10" t="str">
         <x:v>分析：優先向設備客戶確認先進邏輯與記憶體新增設備的認證、拉貨時間及每台設備電源含量，再決定產能與備料。HBM 封裝廠開幕本身，無法證明 AEIS 獲單或收入增加。</x:v>
       </x:c>
-      <x:c r="V4" s="3" t="e">
+      <x:c r="V4" s="10" t="e">
         <x:f>HYPERLINK("https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf","https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf, friendlyName=https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="72" hidden="0" customHeight="1">
-      <x:c r="A5" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B5" s="8" t="d">
+      <x:c r="A5" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B5" s="13" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C5" s="3" t="str">
+      <x:c r="C5" s="10" t="str">
         <x:v>2026-10-17:12</x:v>
       </x:c>
-      <x:c r="D5" s="3" t="str">
+      <x:c r="D5" s="10" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E5" s="3" t="str">
+      <x:c r="E5" s="10" t="str">
         <x:v>AI 半導體；HBM；先進封裝；測試</x:v>
       </x:c>
-      <x:c r="F5" s="3" t="str">
+      <x:c r="F5" s="10" t="str">
         <x:v>毛利率</x:v>
       </x:c>
-      <x:c r="G5" s="3" t="str">
+      <x:c r="G5" s="10" t="str">
         <x:v>公司實績</x:v>
       </x:c>
-      <x:c r="H5" s="3" t="str">
+      <x:c r="H5" s="10" t="str">
         <x:v>2026 Q3</x:v>
       </x:c>
-      <x:c r="I5" s="11" t="n">
+      <x:c r="I5" s="19" t="n">
         <x:v>0.664</x:v>
       </x:c>
-      <x:c r="J5" s="3" t="str">
+      <x:c r="J5" s="10" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="K5" s="3" t="str"/>
-      <x:c r="L5" s="11"/>
-      <x:c r="M5" s="3" t="str">
+      <x:c r="K5" s="10" t="str"/>
+      <x:c r="L5" s="19"/>
+      <x:c r="M5" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N5" s="10"/>
-      <x:c r="O5" s="10"/>
-      <x:c r="P5" s="9"/>
-      <x:c r="Q5" s="9"/>
-      <x:c r="R5" s="10"/>
-      <x:c r="S5" s="3" t="str">
+      <x:c r="N5" s="18"/>
+      <x:c r="O5" s="18"/>
+      <x:c r="P5" s="17"/>
+      <x:c r="Q5" s="17"/>
+      <x:c r="R5" s="18"/>
+      <x:c r="S5" s="10" t="str">
         <x:v>本期值及公布增幅已核對；本表未收錄可比基期</x:v>
       </x:c>
-      <x:c r="T5" s="3" t="str">
+      <x:c r="T5" s="10" t="str">
         <x:v>TSMC</x:v>
       </x:c>
-      <x:c r="U5" s="3" t="str">
+      <x:c r="U5" s="10" t="str">
         <x:v>分析：優先向設備客戶確認先進邏輯與記憶體新增設備的認證、拉貨時間及每台設備電源含量，再決定產能與備料。HBM 封裝廠開幕本身，無法證明 AEIS 獲單或收入增加。</x:v>
       </x:c>
-      <x:c r="V5" s="3" t="e">
+      <x:c r="V5" s="10" t="e">
         <x:f>HYPERLINK("https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf","https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf, friendlyName=https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="100.80000305175781" hidden="0" customHeight="1">
-      <x:c r="A6" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="d">
+      <x:c r="A6" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C6" s="3" t="str">
+      <x:c r="C6" s="10" t="str">
         <x:v>2026-10-17:13</x:v>
       </x:c>
-      <x:c r="D6" s="3" t="str">
+      <x:c r="D6" s="10" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E6" s="3" t="str">
+      <x:c r="E6" s="10" t="str">
         <x:v>AI 資料中心；伺服器；電源；液冷</x:v>
       </x:c>
-      <x:c r="F6" s="3" t="str">
+      <x:c r="F6" s="10" t="str">
         <x:v>電源櫃額定能力</x:v>
       </x:c>
-      <x:c r="G6" s="3" t="str">
+      <x:c r="G6" s="10" t="str">
         <x:v>產品規格</x:v>
       </x:c>
-      <x:c r="H6" s="3" t="str">
+      <x:c r="H6" s="10" t="str">
         <x:v>OCP 2026 展示</x:v>
       </x:c>
-      <x:c r="I6" s="9" t="n">
+      <x:c r="I6" s="17" t="n">
         <x:v>660</x:v>
       </x:c>
-      <x:c r="J6" s="3" t="str">
+      <x:c r="J6" s="10" t="str">
         <x:v>kW</x:v>
       </x:c>
-      <x:c r="K6" s="3" t="str"/>
-      <x:c r="L6" s="9"/>
-      <x:c r="M6" s="3" t="str">
+      <x:c r="K6" s="10" t="str"/>
+      <x:c r="L6" s="17"/>
+      <x:c r="M6" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N6" s="10"/>
-      <x:c r="O6" s="10"/>
-      <x:c r="P6" s="9"/>
-      <x:c r="Q6" s="9"/>
-      <x:c r="R6" s="10"/>
-      <x:c r="S6" s="3" t="str">
+      <x:c r="N6" s="18"/>
+      <x:c r="O6" s="18"/>
+      <x:c r="P6" s="17"/>
+      <x:c r="Q6" s="17"/>
+      <x:c r="R6" s="18"/>
+      <x:c r="S6" s="10" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T6" s="3" t="str">
+      <x:c r="T6" s="10" t="str">
         <x:v>Delta</x:v>
       </x:c>
-      <x:c r="U6" s="3" t="str">
+      <x:c r="U6" s="10" t="str">
         <x:v>分析：應由雲端與 ODM 的認證時程往回排工程資源，確認功率密度、效率、可靠度、備援及供應責任。投資評估需要每櫃電源價值、量產毛利與營運資金，現有公告沒有這些可計算資料。</x:v>
       </x:c>
-      <x:c r="V6" s="3" t="e">
+      <x:c r="V6" s="10" t="e">
         <x:f>HYPERLINK("https://www.prnewswire.com/news-releases/delta-highlights-collaboration-with-nvidia-in-advancing-energy-efficient-800-vdc-power-and-cooling-solutions-for-ai-data-centers-at-ocp-global-summit-2026-302909912.html","https://www.prnewswire.com/news-releases/delta-highlights-collaboration-with-nvidia-in-advancing-energy-efficient-800-vdc-power-and-cooling-solutions-for-ai-data-centers-at-ocp-global-summit-2026-302909912.html")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://www.prnewswire.com/news-releases/delta-highlights-collaboration-with-nvidia-in-advancing-energy-efficient-800-vdc-power-and-cooling-solutions-for-ai-data-centers-at-ocp-global-summit-2026-302909912.html, friendlyName=https://www.prnewswire.com/news-releases/delta-highlights-collaboration-with-nvidia-in-advancing-energy-efficient-800-vdc-power-and-cooling-solutions-for-ai-data-centers-at-ocp-global-summit-2026-302909912.html</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="100.80000305175781" hidden="0" customHeight="1">
-      <x:c r="A7" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B7" s="8" t="d">
+      <x:c r="A7" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B7" s="13" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C7" s="3" t="str">
+      <x:c r="C7" s="10" t="str">
         <x:v>2026-10-17:13</x:v>
       </x:c>
-      <x:c r="D7" s="3" t="str">
+      <x:c r="D7" s="10" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E7" s="3" t="str">
+      <x:c r="E7" s="10" t="str">
         <x:v>AI 資料中心；伺服器；電源；液冷</x:v>
       </x:c>
-      <x:c r="F7" s="3" t="str">
+      <x:c r="F7" s="10" t="str">
         <x:v>備援額定能力</x:v>
       </x:c>
-      <x:c r="G7" s="3" t="str">
+      <x:c r="G7" s="10" t="str">
         <x:v>產品規格</x:v>
       </x:c>
-      <x:c r="H7" s="3" t="str">
+      <x:c r="H7" s="10" t="str">
         <x:v>OCP 2026 展示</x:v>
       </x:c>
-      <x:c r="I7" s="9" t="n">
+      <x:c r="I7" s="17" t="n">
         <x:v>480</x:v>
       </x:c>
-      <x:c r="J7" s="3" t="str">
+      <x:c r="J7" s="10" t="str">
         <x:v>kW</x:v>
       </x:c>
-      <x:c r="K7" s="3" t="str"/>
-      <x:c r="L7" s="9"/>
-      <x:c r="M7" s="3" t="str">
+      <x:c r="K7" s="10" t="str"/>
+      <x:c r="L7" s="17"/>
+      <x:c r="M7" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N7" s="10"/>
-      <x:c r="O7" s="10"/>
-      <x:c r="P7" s="9"/>
-      <x:c r="Q7" s="9"/>
-      <x:c r="R7" s="10"/>
-      <x:c r="S7" s="3" t="str">
+      <x:c r="N7" s="18"/>
+      <x:c r="O7" s="18"/>
+      <x:c r="P7" s="17"/>
+      <x:c r="Q7" s="17"/>
+      <x:c r="R7" s="18"/>
+      <x:c r="S7" s="10" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T7" s="3" t="str">
+      <x:c r="T7" s="10" t="str">
         <x:v>Delta</x:v>
       </x:c>
-      <x:c r="U7" s="3" t="str">
+      <x:c r="U7" s="10" t="str">
         <x:v>分析：應由雲端與 ODM 的認證時程往回排工程資源，確認功率密度、效率、可靠度、備援及供應責任。投資評估需要每櫃電源價值、量產毛利與營運資金，現有公告沒有這些可計算資料。</x:v>
       </x:c>
-      <x:c r="V7" s="3" t="e">
+      <x:c r="V7" s="10" t="e">
         <x:f>HYPERLINK("https://www.prnewswire.com/news-releases/delta-highlights-collaboration-with-nvidia-in-advancing-energy-efficient-800-vdc-power-and-cooling-solutions-for-ai-data-centers-at-ocp-global-summit-2026-302909912.html","https://www.prnewswire.com/news-releases/delta-highlights-collaboration-with-nvidia-in-advancing-energy-efficient-800-vdc-power-and-cooling-solutions-for-ai-data-centers-at-ocp-global-summit-2026-302909912.html")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://www.prnewswire.com/news-releases/delta-highlights-collaboration-with-nvidia-in-advancing-energy-efficient-800-vdc-power-and-cooling-solutions-for-ai-data-centers-at-ocp-global-summit-2026-302909912.html, friendlyName=https://www.prnewswire.com/news-releases/delta-highlights-collaboration-with-nvidia-in-advancing-energy-efficient-800-vdc-power-and-cooling-solutions-for-ai-data-centers-at-ocp-global-summit-2026-302909912.html</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A8" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B8" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="str">
+      <x:c r="A8" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B8" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="str">
         <x:v>2026-10-17:14</x:v>
       </x:c>
-      <x:c r="D8" s="3" t="str">
+      <x:c r="D8" s="10" t="str">
         <x:v>台灣</x:v>
       </x:c>
-      <x:c r="E8" s="3" t="str">
+      <x:c r="E8" s="10" t="str">
         <x:v>玻璃基板；光通訊；先進封裝</x:v>
       </x:c>
-      <x:c r="F8" s="3" t="str">
+      <x:c r="F8" s="10" t="str">
         <x:v>純面板營收占比目標</x:v>
       </x:c>
-      <x:c r="G8" s="3" t="str">
+      <x:c r="G8" s="10" t="str">
         <x:v>公司目標</x:v>
       </x:c>
-      <x:c r="H8" s="3" t="str">
+      <x:c r="H8" s="10" t="str">
         <x:v>2030</x:v>
       </x:c>
-      <x:c r="I8" s="11" t="n">
+      <x:c r="I8" s="19" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="J8" s="3" t="str">
+      <x:c r="J8" s="10" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="K8" s="3" t="str"/>
-      <x:c r="L8" s="11"/>
-      <x:c r="M8" s="3" t="str">
+      <x:c r="K8" s="10" t="str"/>
+      <x:c r="L8" s="19"/>
+      <x:c r="M8" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N8" s="10"/>
-      <x:c r="O8" s="10"/>
-      <x:c r="P8" s="9"/>
-      <x:c r="Q8" s="9"/>
-      <x:c r="R8" s="10"/>
-      <x:c r="S8" s="3" t="str">
+      <x:c r="N8" s="18"/>
+      <x:c r="O8" s="18"/>
+      <x:c r="P8" s="17"/>
+      <x:c r="Q8" s="17"/>
+      <x:c r="R8" s="18"/>
+      <x:c r="S8" s="10" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T8" s="3" t="str">
+      <x:c r="T8" s="10" t="str">
         <x:v>AUO 董事長，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U8" s="3" t="str">
+      <x:c r="U8" s="10" t="str">
         <x:v>分析：先辨識新材料製程使用哪些設備、是否增加電源控制要求，再決定工程投入。零組件轉型可能形成設備需求，現階段未有可量化的 AEIS 訂單或資本支出影響。</x:v>
       </x:c>
-      <x:c r="V8" s="3" t="e">
+      <x:c r="V8" s="10" t="e">
         <x:f>HYPERLINK("https://www.cna.com.tw/news/afe/202610170118.aspx","https://www.cna.com.tw/news/afe/202610170118.aspx")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://www.cna.com.tw/news/afe/202610170118.aspx, friendlyName=https://www.cna.com.tw/news/afe/202610170118.aspx</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="72" hidden="0" customHeight="1">
-      <x:c r="A9" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B9" s="8" t="d">
+      <x:c r="A9" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B9" s="13" t="d">
         <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C9" s="3" t="str">
+      <x:c r="C9" s="10" t="str">
         <x:v>2026-10-17:15</x:v>
       </x:c>
-      <x:c r="D9" s="3" t="str">
+      <x:c r="D9" s="10" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E9" s="3" t="str">
+      <x:c r="E9" s="10" t="str">
         <x:v>終端 AI；PC；IC 設計；封裝</x:v>
       </x:c>
-      <x:c r="F9" s="3" t="str">
+      <x:c r="F9" s="10" t="str">
         <x:v>最高統一記憶體規格</x:v>
       </x:c>
-      <x:c r="G9" s="3" t="str">
+      <x:c r="G9" s="10" t="str">
         <x:v>產品規格</x:v>
       </x:c>
-      <x:c r="H9" s="3" t="str">
+      <x:c r="H9" s="10" t="str">
         <x:v>2026-10-16 發布</x:v>
       </x:c>
-      <x:c r="I9" s="9" t="n">
+      <x:c r="I9" s="17" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="J9" s="3" t="str">
+      <x:c r="J9" s="10" t="str">
         <x:v>GB</x:v>
       </x:c>
-      <x:c r="K9" s="3" t="str"/>
-      <x:c r="L9" s="9"/>
-      <x:c r="M9" s="3" t="str">
+      <x:c r="K9" s="10" t="str"/>
+      <x:c r="L9" s="17"/>
+      <x:c r="M9" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N9" s="10"/>
-      <x:c r="O9" s="10"/>
-      <x:c r="P9" s="9"/>
-      <x:c r="Q9" s="9"/>
-      <x:c r="R9" s="10"/>
-      <x:c r="S9" s="3" t="str">
+      <x:c r="N9" s="18"/>
+      <x:c r="O9" s="18"/>
+      <x:c r="P9" s="17"/>
+      <x:c r="Q9" s="17"/>
+      <x:c r="R9" s="18"/>
+      <x:c r="S9" s="10" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T9" s="3" t="str">
+      <x:c r="T9" s="10" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
-      <x:c r="U9" s="3" t="str">
+      <x:c r="U9" s="10" t="str">
         <x:v>分析：分別追蹤前段設備電源、封裝設備及 PC 系統電源的可服務範圍。新品上市尚不足以調高供應量，應等待通路售出、企業導入、退貨率與平台毛利。</x:v>
       </x:c>
-      <x:c r="V9" s="3" t="e">
+      <x:c r="V9" s="10" t="e">
         <x:f>HYPERLINK("https://nvidianews.nvidia.com/news/nvidia-rtx-spark-pcs-available-today-a-new-beginning-for-windows-pcs","https://nvidianews.nvidia.com/news/nvidia-rtx-spark-pcs-available-today-a-new-beginning-for-windows-pcs")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://nvidianews.nvidia.com/news/nvidia-rtx-spark-pcs-available-today-a-new-beginning-for-windows-pcs, friendlyName=https://nvidianews.nvidia.com/news/nvidia-rtx-spark-pcs-available-today-a-new-beginning-for-windows-pcs</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A10" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B10" s="8" t="d">
+      <x:c r="A10" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B10" s="13" t="d">
         <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C10" s="3" t="str">
+      <x:c r="C10" s="10" t="str">
         <x:v>2026-10-17:4</x:v>
       </x:c>
-      <x:c r="D10" s="3" t="str">
+      <x:c r="D10" s="10" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E10" s="3" t="str">
+      <x:c r="E10" s="10" t="str">
         <x:v>海外工業園區；電子供應鏈</x:v>
       </x:c>
-      <x:c r="F10" s="3" t="str">
+      <x:c r="F10" s="10" t="str">
         <x:v>每座園區估算下限</x:v>
       </x:c>
-      <x:c r="G10" s="3" t="str">
+      <x:c r="G10" s="10" t="str">
         <x:v>規劃估算</x:v>
       </x:c>
-      <x:c r="H10" s="3" t="str">
+      <x:c r="H10" s="10" t="str">
         <x:v>規劃期未定</x:v>
       </x:c>
-      <x:c r="I10" s="9" t="n">
+      <x:c r="I10" s="17" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="J10" s="3" t="str">
+      <x:c r="J10" s="10" t="str">
         <x:v>USD billion</x:v>
       </x:c>
-      <x:c r="K10" s="3" t="str"/>
-      <x:c r="L10" s="9"/>
-      <x:c r="M10" s="3" t="str">
+      <x:c r="K10" s="10" t="str"/>
+      <x:c r="L10" s="17"/>
+      <x:c r="M10" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N10" s="10"/>
-      <x:c r="O10" s="10"/>
-      <x:c r="P10" s="9"/>
-      <x:c r="Q10" s="9"/>
-      <x:c r="R10" s="10"/>
-      <x:c r="S10" s="3" t="str">
+      <x:c r="N10" s="18"/>
+      <x:c r="O10" s="18"/>
+      <x:c r="P10" s="17"/>
+      <x:c r="Q10" s="17"/>
+      <x:c r="R10" s="18"/>
+      <x:c r="S10" s="10" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T10" s="3" t="str">
+      <x:c r="T10" s="10" t="str">
         <x:v>經濟部，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U10" s="3" t="str">
+      <x:c r="U10" s="10" t="str">
         <x:v>大型客戶在美國蓋廠，只完成供應鏈在地化的一部分。對中小供應商，關鍵是園區能否提供穩定訂單、共用設施與可負擔的資金，而不只是一塊海外土地。</x:v>
       </x:c>
-      <x:c r="V10" s="3" t="e">
+      <x:c r="V10" s="10" t="e">
         <x:f>HYPERLINK("https://www.cna.com.tw/news/afe/202610160128.aspx","https://www.cna.com.tw/news/afe/202610160128.aspx")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://www.cna.com.tw/news/afe/202610160128.aspx, friendlyName=https://www.cna.com.tw/news/afe/202610160128.aspx</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="43.20000076293945" hidden="0" customHeight="1">
-      <x:c r="A11" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B11" s="8" t="d">
+      <x:c r="A11" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B11" s="13" t="d">
         <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C11" s="3" t="str">
+      <x:c r="C11" s="10" t="str">
         <x:v>2026-10-17:4</x:v>
       </x:c>
-      <x:c r="D11" s="3" t="str">
+      <x:c r="D11" s="10" t="str">
         <x:v>台灣；美國</x:v>
       </x:c>
-      <x:c r="E11" s="3" t="str">
+      <x:c r="E11" s="10" t="str">
         <x:v>海外工業園區；電子供應鏈</x:v>
       </x:c>
-      <x:c r="F11" s="3" t="str">
+      <x:c r="F11" s="10" t="str">
         <x:v>每座園區估算上限</x:v>
       </x:c>
-      <x:c r="G11" s="3" t="str">
+      <x:c r="G11" s="10" t="str">
         <x:v>規劃估算</x:v>
       </x:c>
-      <x:c r="H11" s="3" t="str">
+      <x:c r="H11" s="10" t="str">
         <x:v>規劃期未定</x:v>
       </x:c>
-      <x:c r="I11" s="9" t="n">
+      <x:c r="I11" s="17" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="J11" s="3" t="str">
+      <x:c r="J11" s="10" t="str">
         <x:v>USD billion</x:v>
       </x:c>
-      <x:c r="K11" s="3" t="str"/>
-      <x:c r="L11" s="9"/>
-      <x:c r="M11" s="3" t="str">
+      <x:c r="K11" s="10" t="str"/>
+      <x:c r="L11" s="17"/>
+      <x:c r="M11" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N11" s="10"/>
-      <x:c r="O11" s="10"/>
-      <x:c r="P11" s="9"/>
-      <x:c r="Q11" s="9"/>
-      <x:c r="R11" s="10"/>
-      <x:c r="S11" s="3" t="str">
+      <x:c r="N11" s="18"/>
+      <x:c r="O11" s="18"/>
+      <x:c r="P11" s="17"/>
+      <x:c r="Q11" s="17"/>
+      <x:c r="R11" s="18"/>
+      <x:c r="S11" s="10" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T11" s="3" t="str">
+      <x:c r="T11" s="10" t="str">
         <x:v>經濟部，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U11" s="3" t="str">
+      <x:c r="U11" s="10" t="str">
         <x:v>大型客戶在美國蓋廠，只完成供應鏈在地化的一部分。對中小供應商，關鍵是園區能否提供穩定訂單、共用設施與可負擔的資金，而不只是一塊海外土地。</x:v>
       </x:c>
-      <x:c r="V11" s="3" t="e">
+      <x:c r="V11" s="10" t="e">
         <x:f>HYPERLINK("https://www.cna.com.tw/news/afe/202610160128.aspx","https://www.cna.com.tw/news/afe/202610160128.aspx")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://www.cna.com.tw/news/afe/202610160128.aspx, friendlyName=https://www.cna.com.tw/news/afe/202610160128.aspx</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="72" hidden="0" customHeight="1">
-      <x:c r="A12" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B12" s="8" t="d">
+      <x:c r="A12" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="d">
         <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C12" s="3" t="str">
+      <x:c r="C12" s="10" t="str">
         <x:v>2026-10-17:11</x:v>
       </x:c>
-      <x:c r="D12" s="3" t="str">
+      <x:c r="D12" s="10" t="str">
         <x:v>台灣</x:v>
       </x:c>
-      <x:c r="E12" s="3" t="str">
+      <x:c r="E12" s="10" t="str">
         <x:v>總體經濟；AI 投資</x:v>
       </x:c>
-      <x:c r="F12" s="3" t="str">
+      <x:c r="F12" s="10" t="str">
         <x:v>2026 年 GDP 成長預測</x:v>
       </x:c>
-      <x:c r="G12" s="3" t="str">
+      <x:c r="G12" s="10" t="str">
         <x:v>預測</x:v>
       </x:c>
-      <x:c r="H12" s="3" t="str">
+      <x:c r="H12" s="10" t="str">
         <x:v>2026 全年，2026-10 預測版</x:v>
       </x:c>
-      <x:c r="I12" s="11" t="n">
+      <x:c r="I12" s="19" t="n">
         <x:v>0.1216</x:v>
       </x:c>
-      <x:c r="J12" s="3" t="str">
+      <x:c r="J12" s="10" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="K12" s="3" t="str">
+      <x:c r="K12" s="10" t="str">
         <x:v>2026 全年，2026-07 預測版</x:v>
       </x:c>
-      <x:c r="L12" s="11" t="n">
+      <x:c r="L12" s="19" t="n">
         <x:v>0.1035</x:v>
       </x:c>
-      <x:c r="M12" s="3" t="str">
+      <x:c r="M12" s="10" t="str">
         <x:v>預測修訂</x:v>
       </x:c>
-      <x:c r="N12" s="10"/>
-      <x:c r="O12" s="10"/>
-      <x:c r="P12" s="9"/>
-      <x:c r="Q12" s="9" t="n">
+      <x:c r="N12" s="18"/>
+      <x:c r="O12" s="18"/>
+      <x:c r="P12" s="17"/>
+      <x:c r="Q12" s="17" t="n">
         <x:f>(I12-L12)*100</x:f>
         <x:v>1.8100000000000005</x:v>
       </x:c>
-      <x:c r="R12" s="10"/>
-      <x:c r="S12" s="3" t="str">
+      <x:c r="R12" s="18"/>
+      <x:c r="S12" s="10" t="str">
         <x:v>已揭露</x:v>
       </x:c>
-      <x:c r="T12" s="3" t="str">
+      <x:c r="T12" s="10" t="str">
         <x:v>CIER</x:v>
       </x:c>
-      <x:c r="U12" s="3" t="str">
+      <x:c r="U12" s="10" t="str">
         <x:v>這份預測的重點是 AI 硬體需求如何傳到投資與消費。分析時仍要分清：少數出口產業的強勁成長、整體 GDP，以及每個人的收入感受，三者不會等比例變動。</x:v>
       </x:c>
-      <x:c r="V12" s="3" t="e">
+      <x:c r="V12" s="10" t="e">
         <x:f>HYPERLINK("https://www.cier.edu.tw/eco/2026%E5%B9%B4%E7%AC%AC4%E5%AD%A3%E8%87%BA%E7%81%A3%E7%B6%93%E6%BF%9F%E9%A0%90%E6%B8%AC/","https://www.cier.edu.tw/eco/2026%E5%B9%B4%E7%AC%AC4%E5%AD%A3%E8%87%BA%E7%81%A3%E7%B6%93%E6%BF%9F%E9%A0%90%E6%B8%AC/")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://www.cier.edu.tw/eco/2026%E5%B9%B4%E7%AC%AC4%E5%AD%A3%E8%87%BA%E7%81%A3%E7%B6%93%E6%BF%9F%E9%A0%90%E6%B8%AC/, friendlyName=https://www.cier.edu.tw/eco/2026%E5%B9%B4%E7%AC%AC4%E5%AD%A3%E8%87%BA%E7%81%A3%E7%B6%93%E6%BF%9F%E9%A0%90%E6%B8%AC/</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="72" hidden="0" customHeight="1">
-      <x:c r="A13" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B13" s="8" t="d">
+      <x:c r="A13" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="d">
         <x:v>2026-10-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C13" s="3" t="str">
+      <x:c r="C13" s="10" t="str">
         <x:v>2026-10-17:18</x:v>
       </x:c>
-      <x:c r="D13" s="3" t="str">
+      <x:c r="D13" s="10" t="str">
         <x:v>越南</x:v>
       </x:c>
-      <x:c r="E13" s="3" t="str">
+      <x:c r="E13" s="10" t="str">
         <x:v>AI 資料中心；電源；能源</x:v>
       </x:c>
-      <x:c r="F13" s="3" t="str">
+      <x:c r="F13" s="10" t="str">
         <x:v>既有資料中心投資計畫</x:v>
       </x:c>
-      <x:c r="G13" s="3" t="str">
+      <x:c r="G13" s="10" t="str">
         <x:v>既有規劃</x:v>
       </x:c>
-      <x:c r="H13" s="3" t="str">
+      <x:c r="H13" s="10" t="str">
         <x:v>2026-03 公布，2026-10 電價追蹤</x:v>
       </x:c>
-      <x:c r="I13" s="9" t="n">
+      <x:c r="I13" s="17" t="n">
         <x:v>2.1</x:v>
       </x:c>
-      <x:c r="J13" s="3" t="str">
+      <x:c r="J13" s="10" t="str">
         <x:v>USD billion</x:v>
       </x:c>
-      <x:c r="K13" s="3" t="str"/>
-      <x:c r="L13" s="9"/>
-      <x:c r="M13" s="3" t="str">
+      <x:c r="K13" s="10" t="str"/>
+      <x:c r="L13" s="17"/>
+      <x:c r="M13" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N13" s="10"/>
-      <x:c r="O13" s="10"/>
-      <x:c r="P13" s="9"/>
-      <x:c r="Q13" s="9"/>
-      <x:c r="R13" s="10"/>
-      <x:c r="S13" s="3" t="str">
+      <x:c r="N13" s="18"/>
+      <x:c r="O13" s="18"/>
+      <x:c r="P13" s="17"/>
+      <x:c r="Q13" s="17"/>
+      <x:c r="R13" s="18"/>
+      <x:c r="S13" s="10" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T13" s="3" t="str">
+      <x:c r="T13" s="10" t="str">
         <x:v>AIC / KBC，由 TNGlobal 報導</x:v>
       </x:c>
-      <x:c r="U13" s="3" t="str">
+      <x:c r="U13" s="10" t="str">
         <x:v>分析：先確認客戶取得的電力條件，再安排機櫃電源工程與交貨。節能、功率密度及可靠度仍有價值，但現有資料不足以估算 AEIS 收入或投資回收。</x:v>
       </x:c>
-      <x:c r="V13" s="3" t="e">
+      <x:c r="V13" s="10" t="e">
         <x:f>HYPERLINK("https://technode.global/2026/10/16/hcmc-seeks-clarification-on-power-price-for-2-1b-ai-data-center/","https://technode.global/2026/10/16/hcmc-seeks-clarification-on-power-price-for-2-1b-ai-data-center/")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://technode.global/2026/10/16/hcmc-seeks-clarification-on-power-price-for-2-1b-ai-data-center/, friendlyName=https://technode.global/2026/10/16/hcmc-seeks-clarification-on-power-price-for-2-1b-ai-data-center/</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="72" hidden="0" customHeight="1">
-      <x:c r="A14" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B14" s="8" t="d">
+      <x:c r="A14" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="d">
         <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C14" s="3" t="str">
+      <x:c r="C14" s="10" t="str">
         <x:v>2026-10-17:19</x:v>
       </x:c>
-      <x:c r="D14" s="3" t="str">
+      <x:c r="D14" s="10" t="str">
         <x:v>馬來西亞；台灣</x:v>
       </x:c>
-      <x:c r="E14" s="3" t="str">
+      <x:c r="E14" s="10" t="str">
         <x:v>半導體；後段封測；設備服務</x:v>
       </x:c>
-      <x:c r="F14" s="3" t="str">
+      <x:c r="F14" s="10" t="str">
         <x:v>活動職缺下限</x:v>
       </x:c>
-      <x:c r="G14" s="3" t="str">
+      <x:c r="G14" s="10" t="str">
         <x:v>超過此數，非實際聘用</x:v>
       </x:c>
-      <x:c r="H14" s="3" t="str">
+      <x:c r="H14" s="10" t="str">
         <x:v>2026-10-14 至 2026-10-17</x:v>
       </x:c>
-      <x:c r="I14" s="9" t="n">
+      <x:c r="I14" s="17" t="n">
         <x:v>1500</x:v>
       </x:c>
-      <x:c r="J14" s="3" t="str">
+      <x:c r="J14" s="10" t="str">
         <x:v>個職缺</x:v>
       </x:c>
-      <x:c r="K14" s="3" t="str"/>
-      <x:c r="L14" s="9"/>
-      <x:c r="M14" s="3" t="str">
+      <x:c r="K14" s="10" t="str"/>
+      <x:c r="L14" s="17"/>
+      <x:c r="M14" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N14" s="10"/>
-      <x:c r="O14" s="10"/>
-      <x:c r="P14" s="9"/>
-      <x:c r="Q14" s="9"/>
-      <x:c r="R14" s="10"/>
-      <x:c r="S14" s="3" t="str">
+      <x:c r="N14" s="18"/>
+      <x:c r="O14" s="18"/>
+      <x:c r="P14" s="17"/>
+      <x:c r="Q14" s="17"/>
+      <x:c r="R14" s="18"/>
+      <x:c r="S14" s="10" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T14" s="3" t="str">
+      <x:c r="T14" s="10" t="str">
         <x:v>主辦活動，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U14" s="3" t="str">
+      <x:c r="U14" s="10" t="str">
         <x:v>分析：區域服務布局應同時評估客戶密度、現場工程人才與維修週轉時間。台馬培訓合作值得追蹤，但本期沒有確認 AEIS 合作、客戶採購或新的工廠投資。</x:v>
       </x:c>
-      <x:c r="V14" s="3" t="e">
+      <x:c r="V14" s="10" t="e">
         <x:f>HYPERLINK("https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side","https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side, friendlyName=https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="72" hidden="0" customHeight="1">
-      <x:c r="A15" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B15" s="8" t="d">
+      <x:c r="A15" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="d">
         <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C15" s="3" t="str">
+      <x:c r="C15" s="10" t="str">
         <x:v>2026-10-17:19</x:v>
       </x:c>
-      <x:c r="D15" s="3" t="str">
+      <x:c r="D15" s="10" t="str">
         <x:v>馬來西亞；台灣</x:v>
       </x:c>
-      <x:c r="E15" s="3" t="str">
+      <x:c r="E15" s="10" t="str">
         <x:v>半導體；後段封測；設備服務</x:v>
       </x:c>
-      <x:c r="F15" s="3" t="str">
+      <x:c r="F15" s="10" t="str">
         <x:v>園區公司數</x:v>
       </x:c>
-      <x:c r="G15" s="3" t="str">
+      <x:c r="G15" s="10" t="str">
         <x:v>官方陳述</x:v>
       </x:c>
-      <x:c r="H15" s="3" t="str">
+      <x:c r="H15" s="10" t="str">
         <x:v>2026-10-16 官員說明</x:v>
       </x:c>
-      <x:c r="I15" s="9" t="n">
+      <x:c r="I15" s="17" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="J15" s="3" t="str">
+      <x:c r="J15" s="10" t="str">
         <x:v>家</x:v>
       </x:c>
-      <x:c r="K15" s="3" t="str"/>
-      <x:c r="L15" s="9"/>
-      <x:c r="M15" s="3" t="str">
+      <x:c r="K15" s="10" t="str"/>
+      <x:c r="L15" s="17"/>
+      <x:c r="M15" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N15" s="10"/>
-      <x:c r="O15" s="10"/>
-      <x:c r="P15" s="9"/>
-      <x:c r="Q15" s="9"/>
-      <x:c r="R15" s="10"/>
-      <x:c r="S15" s="3" t="str">
+      <x:c r="N15" s="18"/>
+      <x:c r="O15" s="18"/>
+      <x:c r="P15" s="17"/>
+      <x:c r="Q15" s="17"/>
+      <x:c r="R15" s="18"/>
+      <x:c r="S15" s="10" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T15" s="3" t="str">
+      <x:c r="T15" s="10" t="str">
         <x:v>雪蘭莪官員，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U15" s="3" t="str">
+      <x:c r="U15" s="10" t="str">
         <x:v>分析：區域服務布局應同時評估客戶密度、現場工程人才與維修週轉時間。台馬培訓合作值得追蹤，但本期沒有確認 AEIS 合作、客戶採購或新的工廠投資。</x:v>
       </x:c>
-      <x:c r="V15" s="3" t="e">
+      <x:c r="V15" s="10" t="e">
         <x:f>HYPERLINK("https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side","https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side, friendlyName=https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="72" hidden="0" customHeight="1">
-      <x:c r="A16" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B16" s="8" t="d">
+      <x:c r="A16" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="d">
         <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C16" s="3" t="str">
+      <x:c r="C16" s="10" t="str">
         <x:v>2026-10-17:19</x:v>
       </x:c>
-      <x:c r="D16" s="3" t="str">
+      <x:c r="D16" s="10" t="str">
         <x:v>馬來西亞；台灣</x:v>
       </x:c>
-      <x:c r="E16" s="3" t="str">
+      <x:c r="E16" s="10" t="str">
         <x:v>半導體；後段封測；設備服務</x:v>
       </x:c>
-      <x:c r="F16" s="3" t="str">
+      <x:c r="F16" s="10" t="str">
         <x:v>園區工程師數</x:v>
       </x:c>
-      <x:c r="G16" s="3" t="str">
+      <x:c r="G16" s="10" t="str">
         <x:v>官方陳述</x:v>
       </x:c>
-      <x:c r="H16" s="3" t="str">
+      <x:c r="H16" s="10" t="str">
         <x:v>2026-10-16 官員說明</x:v>
       </x:c>
-      <x:c r="I16" s="9" t="n">
+      <x:c r="I16" s="17" t="n">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="J16" s="3" t="str">
+      <x:c r="J16" s="10" t="str">
         <x:v>人</x:v>
       </x:c>
-      <x:c r="K16" s="3" t="str"/>
-      <x:c r="L16" s="9"/>
-      <x:c r="M16" s="3" t="str">
+      <x:c r="K16" s="10" t="str"/>
+      <x:c r="L16" s="17"/>
+      <x:c r="M16" s="10" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="N16" s="10"/>
-      <x:c r="O16" s="10"/>
-      <x:c r="P16" s="9"/>
-      <x:c r="Q16" s="9"/>
-      <x:c r="R16" s="10"/>
-      <x:c r="S16" s="3" t="str">
+      <x:c r="N16" s="18"/>
+      <x:c r="O16" s="18"/>
+      <x:c r="P16" s="17"/>
+      <x:c r="Q16" s="17"/>
+      <x:c r="R16" s="18"/>
+      <x:c r="S16" s="10" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T16" s="3" t="str">
+      <x:c r="T16" s="10" t="str">
         <x:v>雪蘭莪官員，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U16" s="3" t="str">
+      <x:c r="U16" s="10" t="str">
         <x:v>分析：區域服務布局應同時評估客戶密度、現場工程人才與維修週轉時間。台馬培訓合作值得追蹤，但本期沒有確認 AEIS 合作、客戶採購或新的工廠投資。</x:v>
       </x:c>
-      <x:c r="V16" s="3" t="e">
+      <x:c r="V16" s="10" t="e">
         <x:f>HYPERLINK("https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side","https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side, friendlyName=https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="72" hidden="0" customHeight="1">
-      <x:c r="A17" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B17" s="8" t="d">
+      <x:c r="A17" s="13" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B17" s="13" t="d">
         <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C17" s="3" t="str">
+      <x:c r="C17" s="10" t="str">
         <x:v>2026-10-17:20</x:v>
       </x:c>
-      <x:c r="D17" s="3" t="str">
+      <x:c r="D17" s="10" t="str">
         <x:v>越南；新加坡</x:v>
       </x:c>
-      <x:c r="E17" s="3" t="str">
+      <x:c r="E17" s="10" t="str">
         <x:v>製造業；外商投資；工業電源</x:v>
       </x:c>
-      <x:c r="F17" s="3" t="str">
+      <x:c r="F17" s="10" t="str">
         <x:v>FDI 實現額估計</x:v>
       </x:c>
-      <x:c r="G17" s="3" t="str">
+      <x:c r="G17" s="10" t="str">
         <x:v>官方估計</x:v>
       </x:c>
-      <x:c r="H17" s="3" t="str">
+      <x:c r="H17" s="10" t="str">
         <x:v>2026-01 至 2026-09</x:v>
       </x:c>
-      <x:c r="I17" s="9" t="n">
+      <x:c r="I17" s="17" t="n">
         <x:v>21.07</x:v>
       </x:c>
-      <x:c r="J17" s="3" t="str">
+      <x:c r="J17" s="10" t="str">
         <x:v>USD billion</x:v>
       </x:c>
-      <x:c r="K17" s="3" t="str">
+      <x:c r="K17" s="10" t="str">
         <x:v>2025-01 至 2025-09</x:v>
       </x:c>
-      <x:c r="L17" s="9"/>
-      <x:c r="M17" s="3" t="str">
+      <x:c r="L17" s="17"/>
+      <x:c r="M17" s="10" t="str">
         <x:v>YoY</x:v>
       </x:c>
-      <x:c r="N17" s="10" t="n">
+      <x:c r="N17" s="18" t="n">
         <x:v>0.121</x:v>
       </x:c>
-      <x:c r="O17" s="10"/>
-      <x:c r="P17" s="9"/>
-      <x:c r="Q17" s="9"/>
-      <x:c r="R17" s="10"/>
-      <x:c r="S17" s="3" t="str">
+      <x:c r="O17" s="18"/>
+      <x:c r="P17" s="17"/>
+      <x:c r="Q17" s="17"/>
+      <x:c r="R17" s="18"/>
+      <x:c r="S17" s="10" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T17" s="3" t="str">
+      <x:c r="T17" s="10" t="str">
         <x:v>越南國家統計局，由政府新聞網公布</x:v>
       </x:c>
-      <x:c r="U17" s="3" t="str">
+      <x:c r="U17" s="10" t="str">
         <x:v>分析：先把投資案對到具名工廠、設備進口、電網接入與驗收，再估在地工業電源及維修需求。全國 FDI 只能提供市場背景，無法直接推成半導體設備或 AEIS 的成長率。</x:v>
       </x:c>
-      <x:c r="V17" s="3" t="e">
+      <x:c r="V17" s="10" t="e">
         <x:f>HYPERLINK("https://en.baochinhphu.vn/viet-nams-gdp-growth-accelerates-to-995-in-q3-111261003093646463.htm","https://en.baochinhphu.vn/viet-nams-gdp-growth-accelerates-to-995-in-q3-111261003093646463.htm")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://en.baochinhphu.vn/viet-nams-gdp-growth-accelerates-to-995-in-q3-111261003093646463.htm, friendlyName=https://en.baochinhphu.vn/viet-nams-gdp-growth-accelerates-to-995-in-q3-111261003093646463.htm</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="72" hidden="0" customHeight="1">
-      <x:c r="A18" s="8" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B18" s="8" t="d">
+      <x:c r="A18" s="14" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B18" s="14" t="d">
         <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C18" s="3" t="str">
+      <x:c r="C18" s="11" t="str">
         <x:v>2026-10-17:20</x:v>
       </x:c>
-      <x:c r="D18" s="3" t="str">
+      <x:c r="D18" s="11" t="str">
         <x:v>越南；新加坡</x:v>
       </x:c>
-      <x:c r="E18" s="3" t="str">
+      <x:c r="E18" s="11" t="str">
         <x:v>製造業；外商投資；工業電源</x:v>
       </x:c>
-      <x:c r="F18" s="3" t="str">
+      <x:c r="F18" s="11" t="str">
         <x:v>總註冊外資</x:v>
       </x:c>
-      <x:c r="G18" s="3" t="str">
+      <x:c r="G18" s="11" t="str">
         <x:v>官方統計</x:v>
       </x:c>
-      <x:c r="H18" s="3" t="str">
+      <x:c r="H18" s="11" t="str">
         <x:v>2026-01 至 2026-09</x:v>
       </x:c>
-      <x:c r="I18" s="9" t="n">
+      <x:c r="I18" s="20" t="n">
         <x:v>50.36</x:v>
       </x:c>
-      <x:c r="J18" s="3" t="str">
+      <x:c r="J18" s="11" t="str">
         <x:v>USD billion</x:v>
       </x:c>
-      <x:c r="K18" s="3" t="str">
+      <x:c r="K18" s="11" t="str">
         <x:v>2025-01 至 2025-09</x:v>
       </x:c>
-      <x:c r="L18" s="9"/>
-      <x:c r="M18" s="3" t="str">
+      <x:c r="L18" s="20"/>
+      <x:c r="M18" s="11" t="str">
         <x:v>YoY</x:v>
       </x:c>
-      <x:c r="N18" s="10" t="n">
+      <x:c r="N18" s="21" t="n">
         <x:v>0.764</x:v>
       </x:c>
-      <x:c r="O18" s="10"/>
-      <x:c r="P18" s="9"/>
-      <x:c r="Q18" s="9"/>
-      <x:c r="R18" s="10"/>
-      <x:c r="S18" s="3" t="str">
+      <x:c r="O18" s="21"/>
+      <x:c r="P18" s="20"/>
+      <x:c r="Q18" s="20"/>
+      <x:c r="R18" s="21"/>
+      <x:c r="S18" s="11" t="str">
         <x:v>未揭露可比基期；不倒推</x:v>
       </x:c>
-      <x:c r="T18" s="3" t="str">
+      <x:c r="T18" s="11" t="str">
         <x:v>越南國家統計局，由政府新聞網公布</x:v>
       </x:c>
-      <x:c r="U18" s="3" t="str">
+      <x:c r="U18" s="11" t="str">
         <x:v>分析：先把投資案對到具名工廠、設備進口、電網接入與驗收，再估在地工業電源及維修需求。全國 FDI 只能提供市場背景，無法直接推成半導體設備或 AEIS 的成長率。</x:v>
       </x:c>
-      <x:c r="V18" s="3" t="e">
+      <x:c r="V18" s="11" t="e">
         <x:f>HYPERLINK("https://en.baochinhphu.vn/viet-nams-gdp-growth-accelerates-to-995-in-q3-111261003093646463.htm","https://en.baochinhphu.vn/viet-nams-gdp-growth-accelerates-to-995-in-q3-111261003093646463.htm")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://en.baochinhphu.vn/viet-nams-gdp-growth-accelerates-to-995-in-q3-111261003093646463.htm, friendlyName=https://en.baochinhphu.vn/viet-nams-gdp-growth-accelerates-to-995-in-q3-111261003093646463.htm</x:v>
       </x:c>
@@ -2059,7 +2123,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4c711fdf80447a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c62177345ab4e9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2084,129 +2148,129 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="3" t="str">
+      <x:c r="A2" s="9" t="str">
         <x:v>閱讀角度</x:v>
       </x:c>
-      <x:c r="B2" s="3" t="str">
+      <x:c r="B2" s="9" t="str">
         <x:v>Advanced Energy Industries (NASDAQ: AEIS)。半導體設備精密電源、資料中心電源、工業客戶與區域服務；影響為編輯分析。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="3" t="str">
+      <x:c r="A3" s="10" t="str">
         <x:v>國家範圍</x:v>
       </x:c>
-      <x:c r="B3" s="3" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>聚焦台灣與東南亞。美國等國家只在直接連結台灣供應鏈時列為關聯地點。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="3" t="str">
+      <x:c r="A4" s="10" t="str">
         <x:v>日期</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="str">
+      <x:c r="B4" s="10" t="str">
         <x:v>刊期與事件日期分欄。週報刊期欄為週起日，個別事件日期請查數值明細與日報。背景資料保留原發布時間。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A5" s="3" t="str">
+      <x:c r="A5" s="10" t="str">
         <x:v>市場動向</x:v>
       </x:c>
-      <x:c r="B5" s="3" t="str">
+      <x:c r="B5" s="10" t="str">
         <x:v>日報每則一列。週報依精選五個主題合併，數值明細保留各事件。市場表連結至日報完整來源，數值表連結至原始數據。下載完整刊期，不受頁面搜尋篩選影響。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="3" t="str">
+      <x:c r="A6" s="10" t="str">
         <x:v>數值與單位</x:v>
       </x:c>
-      <x:c r="B6" s="3" t="str">
+      <x:c r="B6" s="10" t="str">
         <x:v>數值為可計算儲存格，貨幣單位獨立。百分比底層為小數，顯示百分比。不同公司、期間、產品規格及計畫金額不可任意加總。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="3" t="str">
+      <x:c r="A7" s="10" t="str">
         <x:v>Base</x:v>
       </x:c>
-      <x:c r="B7" s="3" t="str">
+      <x:c r="B7" s="10" t="str">
         <x:v>只填來源明示的同口徑基期。缺少則留空並註明，不從已四捨五入成長率反推精確基期。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="3" t="str">
+      <x:c r="A8" s="10" t="str">
         <x:v>YoY / QoQ</x:v>
       </x:c>
-      <x:c r="B8" s="3" t="str">
+      <x:c r="B8" s="10" t="str">
         <x:v>分欄記錄來源公布的年增率與季增率。數值明細可能用不同列表示同一指標的不同比較口徑。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="3" t="str">
+      <x:c r="A9" s="10" t="str">
         <x:v>變動計算</x:v>
       </x:c>
-      <x:c r="B9" s="3" t="str">
+      <x:c r="B9" s="10" t="str">
         <x:v>同口徑且基期可用時，金額變動＝本期減基期；變動率＝本期除基期減一。基期為零時變動率留空。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="3" t="str">
+      <x:c r="A10" s="10" t="str">
         <x:v>百分點</x:v>
       </x:c>
-      <x:c r="B10" s="3" t="str">
+      <x:c r="B10" s="10" t="str">
         <x:v>比例或成長率的修訂以百分點表示。例如 GDP 預測由 10.35% 到 12.16%，增加 1.81 個百分點，並非年增 1.81%。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="3" t="str">
+      <x:c r="A11" s="10" t="str">
         <x:v>資料性質</x:v>
       </x:c>
-      <x:c r="B11" s="3" t="str">
+      <x:c r="B11" s="10" t="str">
         <x:v>區分實績、官方估計、預測、公司目標、規劃與產品規格。規劃不是已實現 FDI，額定能力不是實際用電，職缺不是聘用。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="3" t="str">
+      <x:c r="A12" s="10" t="str">
         <x:v>AEIS 影響</x:v>
       </x:c>
-      <x:c r="B12" s="3" t="str">
+      <x:c r="B12" s="10" t="str">
         <x:v>來源沒有披露 AEIS 訂單或影響金額時保持未知，不以市場增幅直接推算公司收入。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="3" t="str">
+      <x:c r="A13" s="10" t="str">
         <x:v>背景資料</x:v>
       </x:c>
-      <x:c r="B13" s="3" t="str">
+      <x:c r="B13" s="10" t="str">
         <x:v>CoWoS 與美光屬本週追蹤；越南 FDI 於 10/3 發布，非今日新統計。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="57.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A14" s="3" t="str">
+      <x:c r="A14" s="10" t="str">
         <x:v>來源限制</x:v>
       </x:c>
-      <x:c r="B14" s="3" t="str">
+      <x:c r="B14" s="10" t="str">
         <x:v>本期聚焦台灣與東南亞，更新至台北時間 10 月 17 日晚間。CoWoS、美光及越南 10 月 3 日 FDI 資料明列為本週追蹤或區域背景。展示規格、友達目標、園區估算與 GDP 預測均非實際訂單。友達及馬來西亞園區數字依具名採訪；胡志明市電價依專業報導，未取得原始會議文件或最終費率，屬來源受限。AEIS 影響評估為編輯分析，未披露的訂單與金額保持未知。Excel 缺少基期時保留空白及原因，YoY 與百分點分開。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="28.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A15" s="3" t="str">
+      <x:c r="A15" s="10" t="str">
         <x:v>AEIS 業務背景</x:v>
       </x:c>
-      <x:c r="B15" s="3" t="str">
+      <x:c r="B15" s="10" t="str">
         <x:v>https://ir.advancedenergy.com/media/document/fcbde7e4-483b-4dcc-93cc-985a436746b5/assets/2026-09_AEIS_IR_Presentation.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="3" t="str">
+      <x:c r="A16" s="11" t="str">
         <x:v>資料更新</x:v>
       </x:c>
-      <x:c r="B16" s="3" t="d">
+      <x:c r="B16" s="11" t="d">
         <x:v>2026-10-17T10:45:57.185Z</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R459fdd0865084568"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb93ff0d991ad4052"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(news): present industry facts without executive judgments
Retain related Taiwan and Southeast Asia supply-chain reporting, remove editorial recommendations, and leave Excel assessment fields blank for reader analysis.
</commit_message>
<xml_diff>
--- a/docs/exports/day-2026-10-17.xlsx
+++ b/docs/exports/day-2026-10-17.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="市場動向" sheetId="1" r:id="Ree6ca0fc10854099"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="數值明細" sheetId="2" r:id="Rd15165484d5f4a9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="欄位說明" sheetId="3" r:id="R422d59829d4044f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="市場動向" sheetId="1" r:id="R72f3ccba992b4289"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="數值明細" sheetId="2" r:id="R64de6787772c40d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="欄位說明" sheetId="3" r:id="R7194c99e7fef40e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -182,11 +182,11 @@
     <x:tableColumn id="9" name="外商投資 FDI"/>
     <x:tableColumn id="10" name="標題"/>
     <x:tableColumn id="11" name="事件摘要"/>
-    <x:tableColumn id="12" name="業務關聯"/>
-    <x:tableColumn id="13" name="影響評估（分析）"/>
-    <x:tableColumn id="14" name="影響時程"/>
-    <x:tableColumn id="15" name="建議檢查事項"/>
-    <x:tableColumn id="16" name="下一驗證點"/>
+    <x:tableColumn id="12" name="產業關聯"/>
+    <x:tableColumn id="13" name="影響評估（自行填寫）"/>
+    <x:tableColumn id="14" name="已公布時程"/>
+    <x:tableColumn id="15" name="分析備註（自行填寫）"/>
+    <x:tableColumn id="16" name="待確認事項"/>
     <x:tableColumn id="17" name="查證信心"/>
     <x:tableColumn id="18" name="來源類型"/>
     <x:tableColumn id="19" name="完整來源與日報連結"/>
@@ -220,7 +220,7 @@
     <x:tableColumn id="18" name="計算變動率"/>
     <x:tableColumn id="19" name="基期與計算說明"/>
     <x:tableColumn id="20" name="數字歸屬"/>
-    <x:tableColumn id="21" name="營運影響評估（分析）"/>
+    <x:tableColumn id="21" name="影響評估（自行填寫）"/>
     <x:tableColumn id="22" name="來源連結"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -493,19 +493,19 @@
         <x:v>事件摘要</x:v>
       </x:c>
       <x:c r="L1" s="7" t="str">
-        <x:v>業務關聯</x:v>
+        <x:v>產業關聯</x:v>
       </x:c>
       <x:c r="M1" s="7" t="str">
-        <x:v>影響評估（分析）</x:v>
+        <x:v>影響評估（自行填寫）</x:v>
       </x:c>
       <x:c r="N1" s="7" t="str">
-        <x:v>影響時程</x:v>
+        <x:v>已公布時程</x:v>
       </x:c>
       <x:c r="O1" s="7" t="str">
-        <x:v>建議檢查事項</x:v>
+        <x:v>分析備註（自行填寫）</x:v>
       </x:c>
       <x:c r="P1" s="7" t="str">
-        <x:v>下一驗證點</x:v>
+        <x:v>待確認事項</x:v>
       </x:c>
       <x:c r="Q1" s="7" t="str">
         <x:v>查證信心</x:v>
@@ -549,25 +549,21 @@
         <x:v>美商在台廠房開幕，新增金額未披露</x:v>
       </x:c>
       <x:c r="J2" s="9" t="str">
-        <x:v>本週追蹤：AI 晶片供給要同時看 CoWoS、HBM 與後段測試</x:v>
+        <x:v>本週追蹤：台積電 CoWoS 量產與美光台中 HBM 封裝測試廠啟用</x:v>
       </x:c>
       <x:c r="K2" s="9" t="str">
         <x:v>台積電 10 月 15 日法說表示，5 倍光罩尺寸的 CoWoS 已量產；同日美光台中 AATT2 先進封裝測試廠開幕，支援 HBM。這兩項是本週進展，今日整合追蹤，並無新增產能數字。</x:v>
       </x:c>
       <x:c r="L2" s="9" t="str">
-        <x:v>半導體設備精密電源，間接需求</x:v>
-      </x:c>
-      <x:c r="M2" s="9" t="str">
-        <x:v>分析：優先向設備客戶確認先進邏輯與記憶體新增設備的認證、拉貨時間及每台設備電源含量，再決定產能與備料。HBM 封裝廠開幕本身，無法證明 電源供應商 獲單或收入增加。</x:v>
-      </x:c>
+        <x:v>晶圓製造、HBM 與先進封裝測試</x:v>
+      </x:c>
+      <x:c r="M2" s="9" t="str"/>
       <x:c r="N2" s="9" t="str">
-        <x:v>近期認證與中期設備拉貨</x:v>
-      </x:c>
-      <x:c r="O2" s="9" t="str">
-        <x:v>確認設備客戶認證及備料節奏</x:v>
-      </x:c>
+        <x:v>10 月 15 日法說及開幕；量產產出未完整披露</x:v>
+      </x:c>
+      <x:c r="O2" s="9" t="str"/>
       <x:c r="P2" s="9" t="str">
-        <x:v>實際產能、良率、利用率與設備訂單</x:v>
+        <x:v>AATT2 新增 HBM 產出、設備訂單及個別供應商營收未披露</x:v>
       </x:c>
       <x:c r="Q2" s="9" t="str">
         <x:v>高</x:v>
@@ -611,25 +607,21 @@
         <x:v>未披露外商投資金額</x:v>
       </x:c>
       <x:c r="J3" s="10" t="str">
-        <x:v>OCP 台廠展示整機櫃、800 VDC 電源與液冷，量產驗收成為下一關</x:v>
+        <x:v>台廠於聖荷西 OCP 展示整機櫃、800 VDC 電源與液冷</x:v>
       </x:c>
       <x:c r="K3" s="10" t="str">
         <x:v>中央社 10 月 17 日整理 10 月 12 至 15 日於美國加州聖荷西舉辦的 OCP 展會：緯穎、華碩與勤誠等展示下一代伺服器或機櫃，台達電、光寶與康舒展示高壓直流電源及相關方案。台達電 10 月 15 日公司稿列出 800 VDC 電源櫃、備援與液冷產品，展示規格仍需與量產部署分開。</x:v>
       </x:c>
       <x:c r="L3" s="10" t="str">
-        <x:v>資料中心電源直接相關，未證實 電源供應商 新訂單</x:v>
-      </x:c>
-      <x:c r="M3" s="10" t="str">
-        <x:v>分析：應由雲端與 ODM 的認證時程往回排工程資源，確認功率密度、效率、可靠度、備援及供應責任。投資評估需要每櫃電源價值、量產毛利與營運資金，現有公告沒有這些可計算資料。</x:v>
-      </x:c>
+        <x:v>機櫃、電源、備援與液冷產品</x:v>
+      </x:c>
+      <x:c r="M3" s="10" t="str"/>
       <x:c r="N3" s="10" t="str">
-        <x:v>依客戶認證及量產時程</x:v>
-      </x:c>
-      <x:c r="O3" s="10" t="str">
-        <x:v>比較系統整合、效率與服務條件</x:v>
-      </x:c>
+        <x:v>展期 10 月 12 至 15 日；各產品量產時程依廠商披露</x:v>
+      </x:c>
+      <x:c r="O3" s="10" t="str"/>
       <x:c r="P3" s="10" t="str">
-        <x:v>認證、量產訂單與每櫃電源價值</x:v>
+        <x:v>同口徑售價、成本、客戶訂單及實際部署量未披露</x:v>
       </x:c>
       <x:c r="Q3" s="10" t="str">
         <x:v>高</x:v>
@@ -679,19 +671,15 @@
         <x:v>友達董事長彭双浪 10 月 17 日表示，公司在先進封裝將扮演零組件供應者，運用玻璃與 TGV 技術；與康寧合作的技術已有低軌衛星天線應用。MicroLED 光通訊與 CPO 的量產時間估計仍為兩至三年，屬公司展望。</x:v>
       </x:c>
       <x:c r="L4" s="10" t="str">
-        <x:v>新材料設備電源的潛在需求</x:v>
-      </x:c>
-      <x:c r="M4" s="10" t="str">
-        <x:v>分析：先辨識新材料製程使用哪些設備、是否增加電源控制要求，再決定工程投入。零組件轉型可能形成設備需求，現階段未有可量化的 電源供應商 訂單或資本支出影響。</x:v>
-      </x:c>
+        <x:v>玻璃基板、TGV 與光通訊零組件</x:v>
+      </x:c>
+      <x:c r="M4" s="10" t="str"/>
       <x:c r="N4" s="10" t="str">
-        <x:v>光通訊量產展望兩至三年，屬公司估計</x:v>
-      </x:c>
-      <x:c r="O4" s="10" t="str">
-        <x:v>先確認製程與可服務設備</x:v>
-      </x:c>
+        <x:v>2030 年營收組合目標；光通訊量產估兩至三年</x:v>
+      </x:c>
+      <x:c r="O4" s="10" t="str"/>
       <x:c r="P4" s="10" t="str">
-        <x:v>客戶認證、量產良率與新業務收入</x:v>
+        <x:v>新業務獲利、客戶認證及完整逐字稿尚未取得</x:v>
       </x:c>
       <x:c r="Q4" s="10" t="str">
         <x:v>中</x:v>
@@ -741,19 +729,15 @@
         <x:v>NVIDIA 10 月 16 日宣布 RTX Spark Windows 電腦上市，品牌包括華碩、微星及多家國際 PC 廠，採 Grace CPU 與 Blackwell GPU。公司主管向中央社說明聯發科參與 CPU 設計，並使用 CoWoS 封裝；需求與產能判斷仍屬公司說法。</x:v>
       </x:c>
       <x:c r="L5" s="10" t="str">
-        <x:v>PC 電源與製程電源機會需分開</x:v>
-      </x:c>
-      <x:c r="M5" s="10" t="str">
-        <x:v>分析：分別追蹤前段設備電源、封裝設備及 PC 系統電源的可服務範圍。新品上市尚不足以調高供應量，應等待通路售出、企業導入、退貨率與平台毛利。</x:v>
-      </x:c>
+        <x:v>本地 AI 電腦、晶片設計與封裝</x:v>
+      </x:c>
+      <x:c r="M5" s="10" t="str"/>
       <x:c r="N5" s="10" t="str">
-        <x:v>新品上市後數季</x:v>
-      </x:c>
-      <x:c r="O5" s="10" t="str">
-        <x:v>等待售出與企業導入，再調整供應</x:v>
-      </x:c>
+        <x:v>10 月 16 日宣布上市</x:v>
+      </x:c>
+      <x:c r="O5" s="10" t="str"/>
       <x:c r="P5" s="10" t="str">
-        <x:v>出貨、使用率、能耗與退貨率</x:v>
+        <x:v>本期未取得出貨、使用率及完整生命週期成本</x:v>
       </x:c>
       <x:c r="Q5" s="10" t="str">
         <x:v>高</x:v>
@@ -803,19 +787,15 @@
         <x:v>經濟部 10 月 16 日向中央社說明，將與電電公會推動海外產業園區，採業者出資、政府協助模式。龔明鑫專訪提及由德州起步、規劃不只一座；單一園區 20 億至 40 億美元是估算，土地取得細節尚未對外確認。</x:v>
       </x:c>
       <x:c r="L6" s="10" t="str">
-        <x:v>在地服務、庫存與製造成本</x:v>
-      </x:c>
-      <x:c r="M6" s="10" t="str">
-        <x:v>大型客戶在美國蓋廠，只完成供應鏈在地化的一部分。對中小供應商，關鍵是園區能否提供穩定訂單、共用設施與可負擔的資金，而不只是一塊海外土地。</x:v>
-      </x:c>
+        <x:v>海外產業園區與台灣零組件供應鏈</x:v>
+      </x:c>
+      <x:c r="M6" s="10" t="str"/>
       <x:c r="N6" s="10" t="str">
-        <x:v>用地及融資確定後</x:v>
-      </x:c>
-      <x:c r="O6" s="10" t="str">
-        <x:v>以已簽需求檢查布局</x:v>
-      </x:c>
+        <x:v>10 月 16 日說明；土地及動工時程未確認</x:v>
+      </x:c>
+      <x:c r="O6" s="10" t="str"/>
       <x:c r="P6" s="10" t="str">
-        <x:v>融資、土地、入駐名單與動工</x:v>
+        <x:v>開發主體、用地、完整融資及入駐名單尚未確認</x:v>
       </x:c>
       <x:c r="Q6" s="10" t="str">
         <x:v>中</x:v>
@@ -865,19 +845,15 @@
         <x:v>中經院 10 月 16 日公布第四季預測，把 2026 年經濟成長率由 7 月的 10.35% 上修至 12.16%，提高 1.81 個百分點。預估內需貢獻 6.63 個百分點、國外淨需求貢獻 5.53 個百分點；全年數字仍是預測。</x:v>
       </x:c>
       <x:c r="L7" s="10" t="str">
-        <x:v>客戶資本支出與區域服務規劃</x:v>
-      </x:c>
-      <x:c r="M7" s="10" t="str">
-        <x:v>這份預測的重點是 AI 硬體需求如何傳到投資與消費。分析時仍要分清：少數出口產業的強勁成長、整體 GDP，以及每個人的收入感受，三者不會等比例變動。</x:v>
-      </x:c>
+        <x:v>台灣總體經濟及投資、出口統計背景</x:v>
+      </x:c>
+      <x:c r="M7" s="10" t="str"/>
       <x:c r="N7" s="10" t="str">
-        <x:v>2026 年全年預測</x:v>
-      </x:c>
-      <x:c r="O7" s="10" t="str">
-        <x:v>用設備客戶訂單驗證總體展望</x:v>
-      </x:c>
+        <x:v>10 月 16 日公布 2026 年第四季預測</x:v>
+      </x:c>
+      <x:c r="O7" s="10" t="str"/>
       <x:c r="P7" s="10" t="str">
-        <x:v>GDP 實績、民間投資與客戶拉貨</x:v>
+        <x:v>全年 GDP 尚為預測，後續實績可能修訂</x:v>
       </x:c>
       <x:c r="Q7" s="10" t="str">
         <x:v>高</x:v>
@@ -927,19 +903,15 @@
         <x:v>TNGlobal 10 月 16 日報導，胡志明市工業區管理機關在 10 月 15 日經濟會議要求統一 AI 資料中心電價指引。所涉 AIC 與 KBC 計畫早於 3 月公布，總規劃金額 21 億美元；本次新增進展是電價問題，並非新宣布投資。</x:v>
       </x:c>
       <x:c r="L8" s="10" t="str">
-        <x:v>資料中心電源，部署時點風險</x:v>
-      </x:c>
-      <x:c r="M8" s="10" t="str">
-        <x:v>分析：先確認客戶取得的電力條件，再安排機櫃電源工程與交貨。節能、功率密度及可靠度仍有價值，但現有資料不足以估算 電源供應商 收入或投資回收。</x:v>
-      </x:c>
+        <x:v>資料中心電力與越南工業區</x:v>
+      </x:c>
+      <x:c r="M8" s="10" t="str"/>
       <x:c r="N8" s="10" t="str">
-        <x:v>待費率分類與電力合約</x:v>
-      </x:c>
-      <x:c r="O8" s="10" t="str">
-        <x:v>確認電力條件再排工程及交貨</x:v>
-      </x:c>
+        <x:v>10 月 15 日會議、10 月 16 日報導；最終費率未定</x:v>
+      </x:c>
+      <x:c r="O8" s="10" t="str"/>
       <x:c r="P8" s="10" t="str">
-        <x:v>正式費率、融資與上線</x:v>
+        <x:v>原始會議文件、最終費率、用電曲線與電力合約未取得</x:v>
       </x:c>
       <x:c r="Q8" s="10" t="str">
         <x:v>中</x:v>
@@ -989,19 +961,15 @@
         <x:v>中央社 10 月 16 日報導，雪蘭莪相關機構在吉隆坡會展中心（KLCC）主辦的半導體招募活動提供逾 1,500 個職缺，涵蓋設計、軟韌體、製程、設備及廠務。官員表示兩座 IC 設計園區有 20 家公司、409 名工程師，與檳城製造、組裝測試形成互補。</x:v>
       </x:c>
       <x:c r="L9" s="10" t="str">
-        <x:v>區域服務與工程人才，間接相關</x:v>
-      </x:c>
-      <x:c r="M9" s="10" t="str">
-        <x:v>分析：區域服務布局應同時評估客戶密度、現場工程人才與維修週轉時間。台馬培訓合作值得追蹤，但本期沒有確認 電源供應商 合作、客戶採購或新的工廠投資。</x:v>
-      </x:c>
+        <x:v>IC 設計、製程、設備、廠務與封測人才</x:v>
+      </x:c>
+      <x:c r="M9" s="10" t="str"/>
       <x:c r="N9" s="10" t="str">
-        <x:v>當期招募與後續認證</x:v>
-      </x:c>
-      <x:c r="O9" s="10" t="str">
-        <x:v>檢查客戶密度、人才與維修週轉</x:v>
-      </x:c>
+        <x:v>10 月中旬招募；主辦頁起日為 10/14 或 10/15</x:v>
+      </x:c>
+      <x:c r="O9" s="10" t="str"/>
       <x:c r="P9" s="10" t="str">
-        <x:v>聘用、留任與客戶設備認證</x:v>
+        <x:v>實際聘用與留任未披露；園區及計畫數字依官員陳述</x:v>
       </x:c>
       <x:c r="Q9" s="10" t="str">
         <x:v>中</x:v>
@@ -1051,19 +1019,15 @@
         <x:v>越南政府新聞網 10 月 3 日公布的前三季資料顯示，FDI 實現額估 210.7 億美元、年增 12.1%，總註冊外資為 503.6 億美元、年增 76.4%。這是本期新增的區域背景，資料截至 9 月 30 日，並非 10 月 17 日的新統計。</x:v>
       </x:c>
       <x:c r="L10" s="10" t="str">
-        <x:v>在地工業電源與服務的背景指標</x:v>
-      </x:c>
-      <x:c r="M10" s="10" t="str">
-        <x:v>分析：先把投資案對到具名工廠、設備進口、電網接入與驗收，再估在地工業電源及維修需求。全國 FDI 只能提供市場背景，無法直接推成半導體設備或 電源供應商 的成長率。</x:v>
-      </x:c>
+        <x:v>越南製造業投資及外資流量背景</x:v>
+      </x:c>
+      <x:c r="M10" s="10" t="str"/>
       <x:c r="N10" s="10" t="str">
-        <x:v>截至 2026 年 9 月的區域背景</x:v>
-      </x:c>
-      <x:c r="O10" s="10" t="str">
-        <x:v>對到具名廠房與設備採購</x:v>
-      </x:c>
+        <x:v>統計截至 9 月 30 日，10 月 3 日發布</x:v>
+      </x:c>
+      <x:c r="O10" s="10" t="str"/>
       <x:c r="P10" s="10" t="str">
-        <x:v>製造業分項、電網接入與驗收</x:v>
+        <x:v>製造業及資金來源分項未核對官方原表；實現額屬估計</x:v>
       </x:c>
       <x:c r="Q10" s="10" t="str">
         <x:v>中：總量有官方來源，新增分項待核對原表</x:v>
@@ -1107,25 +1071,21 @@
         <x:v>未揭露</x:v>
       </x:c>
       <x:c r="J11" s="11" t="str">
-        <x:v>背景追蹤：工廠 AI 合作延伸到檢測、測試與數位分身，收益仍待驗收</x:v>
+        <x:v>背景追蹤：NVIDIA 公布半導體檢測、測試與工廠 AI 合作</x:v>
       </x:c>
       <x:c r="K11" s="11" t="str">
         <x:v>NVIDIA 10 月 14 日公司稿列出 KLA 檢測、Advantest 測試，以及鴻海、FANUC 等工廠 AI 合作。本期把它作為台灣供應鏈與終端工廠的背景追蹤；各場域地點、全面量產時程與全廠投資報酬未完整公開。</x:v>
       </x:c>
       <x:c r="L11" s="11" t="str">
-        <x:v>工業設備、製程控制及售後服務</x:v>
-      </x:c>
-      <x:c r="M11" s="11" t="str">
-        <x:v>分析：設備與軟體能否改善單一工序，和整廠能否增加可交付產出，是兩個驗收問題。採購前應建立基期，追到良率、停機、返工及現金回收。</x:v>
-      </x:c>
+        <x:v>檢測、測試設備與工廠 AI 軟硬體合作</x:v>
+      </x:c>
+      <x:c r="M11" s="11" t="str"/>
       <x:c r="N11" s="11" t="str">
-        <x:v>試點至量產驗收，時程未完整公開</x:v>
-      </x:c>
-      <x:c r="O11" s="11" t="str">
-        <x:v>先建立基期，再看良品成本與現金回收</x:v>
-      </x:c>
+        <x:v>10 月 14 日公司發布；全面部署時程未完整公開</x:v>
+      </x:c>
+      <x:c r="O11" s="11" t="str"/>
       <x:c r="P11" s="11" t="str">
-        <x:v>具名工廠、同條件數據、驗收與維護成本</x:v>
+        <x:v>具名部署廠址、合約計價與量化全廠收益未完整公開</x:v>
       </x:c>
       <x:c r="Q11" s="11" t="str">
         <x:v>中</x:v>
@@ -1143,7 +1103,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf53f71e68ad1478e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04b8ccfbbe494158"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1241,13 +1201,13 @@
         <x:v>數字歸屬</x:v>
       </x:c>
       <x:c r="U1" s="7" t="str">
-        <x:v>營運影響評估（分析）</x:v>
+        <x:v>影響評估（自行填寫）</x:v>
       </x:c>
       <x:c r="V1" s="7" t="str">
         <x:v>來源連結</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="2" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A2" s="12" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -1298,14 +1258,12 @@
       <x:c r="T2" s="9" t="str">
         <x:v>TSMC</x:v>
       </x:c>
-      <x:c r="U2" s="9" t="str">
-        <x:v>分析：優先向設備客戶確認先進邏輯與記憶體新增設備的認證、拉貨時間及每台設備電源含量，再決定產能與備料。HBM 封裝廠開幕本身，無法證明 電源供應商 獲單或收入增加。</x:v>
-      </x:c>
+      <x:c r="U2" s="9" t="str"/>
       <x:c r="V2" s="9" t="str">
         <x:v>https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="3" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A3" s="13" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -1356,14 +1314,12 @@
       <x:c r="T3" s="10" t="str">
         <x:v>TSMC</x:v>
       </x:c>
-      <x:c r="U3" s="10" t="str">
-        <x:v>分析：優先向設備客戶確認先進邏輯與記憶體新增設備的認證、拉貨時間及每台設備電源含量，再決定產能與備料。HBM 封裝廠開幕本身，無法證明 電源供應商 獲單或收入增加。</x:v>
-      </x:c>
+      <x:c r="U3" s="10" t="str"/>
       <x:c r="V3" s="10" t="str">
         <x:v>https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="4" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A4" s="13" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -1410,14 +1366,12 @@
       <x:c r="T4" s="10" t="str">
         <x:v>TSMC</x:v>
       </x:c>
-      <x:c r="U4" s="10" t="str">
-        <x:v>分析：優先向設備客戶確認先進邏輯與記憶體新增設備的認證、拉貨時間及每台設備電源含量，再決定產能與備料。HBM 封裝廠開幕本身，無法證明 電源供應商 獲單或收入增加。</x:v>
-      </x:c>
+      <x:c r="U4" s="10" t="str"/>
       <x:c r="V4" s="10" t="str">
         <x:v>https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="5" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A5" s="13" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -1464,9 +1418,7 @@
       <x:c r="T5" s="10" t="str">
         <x:v>TSMC</x:v>
       </x:c>
-      <x:c r="U5" s="10" t="str">
-        <x:v>分析：優先向設備客戶確認先進邏輯與記憶體新增設備的認證、拉貨時間及每台設備電源含量，再決定產能與備料。HBM 封裝廠開幕本身，無法證明 電源供應商 獲單或收入增加。</x:v>
-      </x:c>
+      <x:c r="U5" s="10" t="str"/>
       <x:c r="V5" s="10" t="str">
         <x:v>https://investor.tsmc.com/english/encrypt/files/encrypt_file/reports/2026-10/526b65af7305df2dde6b9ece6812b1fdf1e49f9b/3Q26%20EarningsRelease.pdf</x:v>
       </x:c>
@@ -1518,9 +1470,7 @@
       <x:c r="T6" s="10" t="str">
         <x:v>Delta</x:v>
       </x:c>
-      <x:c r="U6" s="10" t="str">
-        <x:v>分析：應由雲端與 ODM 的認證時程往回排工程資源，確認功率密度、效率、可靠度、備援及供應責任。投資評估需要每櫃電源價值、量產毛利與營運資金，現有公告沒有這些可計算資料。</x:v>
-      </x:c>
+      <x:c r="U6" s="10" t="str"/>
       <x:c r="V6" s="10" t="str">
         <x:v>https://www.prnewswire.com/news-releases/delta-highlights-collaboration-with-nvidia-in-advancing-energy-efficient-800-vdc-power-and-cooling-solutions-for-ai-data-centers-at-ocp-global-summit-2026-302909912.html</x:v>
       </x:c>
@@ -1572,14 +1522,12 @@
       <x:c r="T7" s="10" t="str">
         <x:v>Delta</x:v>
       </x:c>
-      <x:c r="U7" s="10" t="str">
-        <x:v>分析：應由雲端與 ODM 的認證時程往回排工程資源，確認功率密度、效率、可靠度、備援及供應責任。投資評估需要每櫃電源價值、量產毛利與營運資金，現有公告沒有這些可計算資料。</x:v>
-      </x:c>
+      <x:c r="U7" s="10" t="str"/>
       <x:c r="V7" s="10" t="str">
         <x:v>https://www.prnewswire.com/news-releases/delta-highlights-collaboration-with-nvidia-in-advancing-energy-efficient-800-vdc-power-and-cooling-solutions-for-ai-data-centers-at-ocp-global-summit-2026-302909912.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="28.799999237060547" hidden="0" customHeight="1">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="13" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -1626,14 +1574,12 @@
       <x:c r="T8" s="10" t="str">
         <x:v>AUO 董事長，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U8" s="10" t="str">
-        <x:v>分析：先辨識新材料製程使用哪些設備、是否增加電源控制要求，再決定工程投入。零組件轉型可能形成設備需求，現階段未有可量化的 電源供應商 訂單或資本支出影響。</x:v>
-      </x:c>
+      <x:c r="U8" s="10" t="str"/>
       <x:c r="V8" s="10" t="str">
         <x:v>https://www.cna.com.tw/news/afe/202610170118.aspx</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="9" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A9" s="13" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -1680,14 +1626,12 @@
       <x:c r="T9" s="10" t="str">
         <x:v>NVIDIA</x:v>
       </x:c>
-      <x:c r="U9" s="10" t="str">
-        <x:v>分析：分別追蹤前段設備電源、封裝設備及 PC 系統電源的可服務範圍。新品上市尚不足以調高供應量，應等待通路售出、企業導入、退貨率與平台毛利。</x:v>
-      </x:c>
+      <x:c r="U9" s="10" t="str"/>
       <x:c r="V9" s="10" t="str">
         <x:v>https://nvidianews.nvidia.com/news/nvidia-rtx-spark-pcs-available-today-a-new-beginning-for-windows-pcs</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="28.799999237060547" hidden="0" customHeight="1">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="13" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -1734,14 +1678,12 @@
       <x:c r="T10" s="10" t="str">
         <x:v>經濟部，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U10" s="10" t="str">
-        <x:v>大型客戶在美國蓋廠，只完成供應鏈在地化的一部分。對中小供應商，關鍵是園區能否提供穩定訂單、共用設施與可負擔的資金，而不只是一塊海外土地。</x:v>
-      </x:c>
+      <x:c r="U10" s="10" t="str"/>
       <x:c r="V10" s="10" t="str">
         <x:v>https://www.cna.com.tw/news/afe/202610160128.aspx</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="28.799999237060547" hidden="0" customHeight="1">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="13" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -1788,14 +1730,12 @@
       <x:c r="T11" s="10" t="str">
         <x:v>經濟部，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U11" s="10" t="str">
-        <x:v>大型客戶在美國蓋廠，只完成供應鏈在地化的一部分。對中小供應商，關鍵是園區能否提供穩定訂單、共用設施與可負擔的資金，而不只是一塊海外土地。</x:v>
-      </x:c>
+      <x:c r="U11" s="10" t="str"/>
       <x:c r="V11" s="10" t="str">
         <x:v>https://www.cna.com.tw/news/afe/202610160128.aspx</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="43.20000076293945" hidden="0" customHeight="1">
+    <x:row r="12" ht="28.799999237060547" hidden="0" customHeight="1">
       <x:c r="A12" s="13" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -1849,9 +1789,7 @@
       <x:c r="T12" s="10" t="str">
         <x:v>CIER</x:v>
       </x:c>
-      <x:c r="U12" s="10" t="str">
-        <x:v>這份預測的重點是 AI 硬體需求如何傳到投資與消費。分析時仍要分清：少數出口產業的強勁成長、整體 GDP，以及每個人的收入感受，三者不會等比例變動。</x:v>
-      </x:c>
+      <x:c r="U12" s="10" t="str"/>
       <x:c r="V12" s="10" t="str">
         <x:v>https://www.cier.edu.tw/eco/2026%E5%B9%B4%E7%AC%AC4%E5%AD%A3%E8%87%BA%E7%81%A3%E7%B6%93%E6%BF%9F%E9%A0%90%E6%B8%AC/</x:v>
       </x:c>
@@ -1903,9 +1841,7 @@
       <x:c r="T13" s="10" t="str">
         <x:v>AIC / KBC，由 TNGlobal 報導</x:v>
       </x:c>
-      <x:c r="U13" s="10" t="str">
-        <x:v>分析：先確認客戶取得的電力條件，再安排機櫃電源工程與交貨。節能、功率密度及可靠度仍有價值，但現有資料不足以估算 電源供應商 收入或投資回收。</x:v>
-      </x:c>
+      <x:c r="U13" s="10" t="str"/>
       <x:c r="V13" s="10" t="str">
         <x:v>https://technode.global/2026/10/16/hcmc-seeks-clarification-on-power-price-for-2-1b-ai-data-center/</x:v>
       </x:c>
@@ -1957,14 +1893,12 @@
       <x:c r="T14" s="10" t="str">
         <x:v>AIC / KBC 計畫，由 TNGlobal 報導</x:v>
       </x:c>
-      <x:c r="U14" s="10" t="str">
-        <x:v>分析：先確認客戶取得的電力條件，再安排機櫃電源工程與交貨。節能、功率密度及可靠度仍有價值，但現有資料不足以估算 電源供應商 收入或投資回收。</x:v>
-      </x:c>
+      <x:c r="U14" s="10" t="str"/>
       <x:c r="V14" s="10" t="str">
         <x:v>https://technode.global/2026/10/16/hcmc-seeks-clarification-on-power-price-for-2-1b-ai-data-center/</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="28.799999237060547" hidden="0" customHeight="1">
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="13" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -2011,14 +1945,12 @@
       <x:c r="T15" s="10" t="str">
         <x:v>主辦活動，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U15" s="10" t="str">
-        <x:v>分析：區域服務布局應同時評估客戶密度、現場工程人才與維修週轉時間。台馬培訓合作值得追蹤，但本期沒有確認 電源供應商 合作、客戶採購或新的工廠投資。</x:v>
-      </x:c>
+      <x:c r="U15" s="10" t="str"/>
       <x:c r="V15" s="10" t="str">
         <x:v>https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="28.799999237060547" hidden="0" customHeight="1">
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="13" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -2065,14 +1997,12 @@
       <x:c r="T16" s="10" t="str">
         <x:v>雪蘭莪官員，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U16" s="10" t="str">
-        <x:v>分析：區域服務布局應同時評估客戶密度、現場工程人才與維修週轉時間。台馬培訓合作值得追蹤，但本期沒有確認 電源供應商 合作、客戶採購或新的工廠投資。</x:v>
-      </x:c>
+      <x:c r="U16" s="10" t="str"/>
       <x:c r="V16" s="10" t="str">
         <x:v>https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="28.799999237060547" hidden="0" customHeight="1">
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="13" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
@@ -2119,9 +2049,7 @@
       <x:c r="T17" s="10" t="str">
         <x:v>雪蘭莪官員，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U17" s="10" t="str">
-        <x:v>分析：區域服務布局應同時評估客戶密度、現場工程人才與維修週轉時間。台馬培訓合作值得追蹤，但本期沒有確認 電源供應商 合作、客戶採購或新的工廠投資。</x:v>
-      </x:c>
+      <x:c r="U17" s="10" t="str"/>
       <x:c r="V17" s="10" t="str">
         <x:v>https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side</x:v>
       </x:c>
@@ -2173,9 +2101,7 @@
       <x:c r="T18" s="10" t="str">
         <x:v>雪蘭莪官員，由 CNA 報導</x:v>
       </x:c>
-      <x:c r="U18" s="10" t="str">
-        <x:v>分析：區域服務布局應同時評估客戶密度、現場工程人才與維修週轉時間。台馬培訓合作值得追蹤，但本期沒有確認 電源供應商 合作、客戶採購或新的工廠投資。</x:v>
-      </x:c>
+      <x:c r="U18" s="10" t="str"/>
       <x:c r="V18" s="10" t="str">
         <x:v>https://money.udn.com/money/story/5599/9819018?from=edn_newestlist_cate_side</x:v>
       </x:c>
@@ -2231,9 +2157,7 @@
       <x:c r="T19" s="10" t="str">
         <x:v>越南國家統計局，由政府新聞網公布</x:v>
       </x:c>
-      <x:c r="U19" s="10" t="str">
-        <x:v>分析：先把投資案對到具名工廠、設備進口、電網接入與驗收，再估在地工業電源及維修需求。全國 FDI 只能提供市場背景，無法直接推成半導體設備或 電源供應商 的成長率。</x:v>
-      </x:c>
+      <x:c r="U19" s="10" t="str"/>
       <x:c r="V19" s="10" t="str">
         <x:v>https://en.baochinhphu.vn/viet-nams-gdp-growth-accelerates-to-995-in-q3-111261003093646463.htm</x:v>
       </x:c>
@@ -2289,9 +2213,7 @@
       <x:c r="T20" s="10" t="str">
         <x:v>越南國家統計局，由政府新聞網公布</x:v>
       </x:c>
-      <x:c r="U20" s="10" t="str">
-        <x:v>分析：先把投資案對到具名工廠、設備進口、電網接入與驗收，再估在地工業電源及維修需求。全國 FDI 只能提供市場背景，無法直接推成半導體設備或 電源供應商 的成長率。</x:v>
-      </x:c>
+      <x:c r="U20" s="10" t="str"/>
       <x:c r="V20" s="10" t="str">
         <x:v>https://en.baochinhphu.vn/viet-nams-gdp-growth-accelerates-to-995-in-q3-111261003093646463.htm</x:v>
       </x:c>
@@ -2343,9 +2265,7 @@
       <x:c r="T21" s="10" t="str">
         <x:v>越南統計資料，由 VnEconomy 轉述</x:v>
       </x:c>
-      <x:c r="U21" s="10" t="str">
-        <x:v>分析：先把投資案對到具名工廠、設備進口、電網接入與驗收，再估在地工業電源及維修需求。全國 FDI 只能提供市場背景，無法直接推成半導體設備或 電源供應商 的成長率。</x:v>
-      </x:c>
+      <x:c r="U21" s="10" t="str"/>
       <x:c r="V21" s="10" t="str">
         <x:v>https://en.vneconomy.vn/vietnams-fdi-attraction-reaches-5036bln-in-9m.htm</x:v>
       </x:c>
@@ -2397,9 +2317,7 @@
       <x:c r="T22" s="11" t="str">
         <x:v>越南統計資料，由 VnEconomy 轉述</x:v>
       </x:c>
-      <x:c r="U22" s="11" t="str">
-        <x:v>分析：先把投資案對到具名工廠、設備進口、電網接入與驗收，再估在地工業電源及維修需求。全國 FDI 只能提供市場背景，無法直接推成半導體設備或 電源供應商 的成長率。</x:v>
-      </x:c>
+      <x:c r="U22" s="11" t="str"/>
       <x:c r="V22" s="11" t="str">
         <x:v>https://en.vneconomy.vn/vietnams-fdi-attraction-reaches-5036bln-in-9m.htm</x:v>
       </x:c>
@@ -2407,7 +2325,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b6c4bef19564039"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc10be2faefcb4669"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2433,10 +2351,10 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>閱讀角度</x:v>
+        <x:v>涵蓋範圍</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>從半導體設備、電源、資料中心與工業供應鏈的經營決策評估市場；影響判斷為編輯分析。</x:v>
+        <x:v>半導體設備、精密電源、資料中心與工業上下游供應鏈。內容整理已公布事實、數據、來源及資料缺口。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -2513,10 +2431,10 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="10" t="str">
-        <x:v>營運影響</x:v>
+        <x:v>自行分析</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
-        <x:v>未披露的訂單或影響金額保持未知，不以市場增幅直接推算個別公司的收入。</x:v>
+        <x:v>影響評估與分析備註欄留白，由讀者填寫。未披露的訂單或影響金額保持未知。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -2532,7 +2450,7 @@
         <x:v>來源限制</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>本期聚焦台灣與東南亞。CoWoS、美光、10 月 14 日工廠 AI 合作及越南 10 月 3 日 FDI 資料明列為追蹤或背景。展示規格、公司目標、園區估算與 GDP 預測均非已完成訂單。友達與馬來西亞園區數字依具名採訪；胡志明市電價缺原始會議文件及最終費率，越南製造業及資金來源分項未核對官方原表，這些部分屬來源受限。營運影響與情境推演為編輯分析，未披露的訂單、基期與影響金額保持未知。 活動地點依主辦資料補充；MSRD 招募起日存在 10/14 與 10/15 兩種主辦頁記載，KLCC 場館則一致。</x:v>
+        <x:v>本期聚焦台灣與東南亞。CoWoS、美光、10 月 14 日工廠 AI 合作及越南 10 月 3 日 FDI 資料明列為追蹤或背景。展示規格、公司目標、園區估算與 GDP 預測均非已完成訂單。友達與馬來西亞園區數字依具名採訪；胡志明市電價缺原始會議文件及最終費率，越南製造業及資金來源分項未核對官方原表，這些部分屬來源受限。未披露的訂單、基期與影響金額保持未知。 活動地點依主辦資料補充；MSRD 招募起日存在 10/14 與 10/15 兩種主辦頁記載，KLCC 場館則一致。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -2548,13 +2466,13 @@
         <x:v>資料更新</x:v>
       </x:c>
       <x:c r="B16" s="11" t="d">
-        <x:v>2026-10-17T11:34:06.828Z</x:v>
+        <x:v>2026-10-17T11:53:49.157Z</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95ec172c6d644ddd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd79b98bf8c6b47cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>